<commit_message>
Show warranty start from first successful activation-code issuance
</commit_message>
<xml_diff>
--- a/public/templates/distribution-import.xlsx
+++ b/public/templates/distribution-import.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اطلاعات" sheetId="1" r:id="Re995621ac4fa461f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنما" sheetId="2" r:id="R0dab36cd426c497c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اطلاعات" sheetId="1" r:id="Rb88640b36f8f42a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنما" sheetId="2" r:id="Redc4a346ee4842a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -295,8 +295,7 @@
     <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="40" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="36" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="36" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="40" customHeight="1">
@@ -331,9 +330,6 @@
         <x:v>نشانی مشتری</x:v>
       </x:c>
       <x:c r="K1" s="6" t="str">
-        <x:v>تاریخ تحویل به مشتری</x:v>
-      </x:c>
-      <x:c r="L1" s="6" t="str">
         <x:v>توضیحات</x:v>
       </x:c>
     </x:row>
@@ -348,8 +344,7 @@
       <x:c r="H2" s="8"/>
       <x:c r="I2" s="7"/>
       <x:c r="J2" s="7"/>
-      <x:c r="K2" s="10"/>
-      <x:c r="L2" s="7"/>
+      <x:c r="K2" s="7"/>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="8"/>
@@ -362,8 +357,7 @@
       <x:c r="H3" s="8"/>
       <x:c r="I3" s="7"/>
       <x:c r="J3" s="7"/>
-      <x:c r="K3" s="10"/>
-      <x:c r="L3" s="7"/>
+      <x:c r="K3" s="7"/>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="8"/>
@@ -376,8 +370,7 @@
       <x:c r="H4" s="8"/>
       <x:c r="I4" s="7"/>
       <x:c r="J4" s="7"/>
-      <x:c r="K4" s="10"/>
-      <x:c r="L4" s="7"/>
+      <x:c r="K4" s="7"/>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="8"/>
@@ -390,8 +383,7 @@
       <x:c r="H5" s="8"/>
       <x:c r="I5" s="7"/>
       <x:c r="J5" s="7"/>
-      <x:c r="K5" s="10"/>
-      <x:c r="L5" s="7"/>
+      <x:c r="K5" s="7"/>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="8"/>
@@ -404,8 +396,7 @@
       <x:c r="H6" s="8"/>
       <x:c r="I6" s="7"/>
       <x:c r="J6" s="7"/>
-      <x:c r="K6" s="10"/>
-      <x:c r="L6" s="7"/>
+      <x:c r="K6" s="7"/>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
       <x:c r="A7" s="8"/>
@@ -418,8 +409,7 @@
       <x:c r="H7" s="8"/>
       <x:c r="I7" s="7"/>
       <x:c r="J7" s="7"/>
-      <x:c r="K7" s="10"/>
-      <x:c r="L7" s="7"/>
+      <x:c r="K7" s="7"/>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="8"/>
@@ -432,8 +422,7 @@
       <x:c r="H8" s="8"/>
       <x:c r="I8" s="7"/>
       <x:c r="J8" s="7"/>
-      <x:c r="K8" s="10"/>
-      <x:c r="L8" s="7"/>
+      <x:c r="K8" s="7"/>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="8"/>
@@ -446,8 +435,7 @@
       <x:c r="H9" s="8"/>
       <x:c r="I9" s="7"/>
       <x:c r="J9" s="7"/>
-      <x:c r="K9" s="10"/>
-      <x:c r="L9" s="7"/>
+      <x:c r="K9" s="7"/>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="8"/>
@@ -460,8 +448,7 @@
       <x:c r="H10" s="8"/>
       <x:c r="I10" s="7"/>
       <x:c r="J10" s="7"/>
-      <x:c r="K10" s="10"/>
-      <x:c r="L10" s="7"/>
+      <x:c r="K10" s="7"/>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="8"/>
@@ -474,8 +461,7 @@
       <x:c r="H11" s="8"/>
       <x:c r="I11" s="7"/>
       <x:c r="J11" s="7"/>
-      <x:c r="K11" s="10"/>
-      <x:c r="L11" s="7"/>
+      <x:c r="K11" s="7"/>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="8"/>
@@ -488,8 +474,7 @@
       <x:c r="H12" s="8"/>
       <x:c r="I12" s="7"/>
       <x:c r="J12" s="7"/>
-      <x:c r="K12" s="10"/>
-      <x:c r="L12" s="7"/>
+      <x:c r="K12" s="7"/>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="8"/>
@@ -502,8 +487,7 @@
       <x:c r="H13" s="8"/>
       <x:c r="I13" s="7"/>
       <x:c r="J13" s="7"/>
-      <x:c r="K13" s="10"/>
-      <x:c r="L13" s="7"/>
+      <x:c r="K13" s="7"/>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="8"/>
@@ -516,8 +500,7 @@
       <x:c r="H14" s="8"/>
       <x:c r="I14" s="7"/>
       <x:c r="J14" s="7"/>
-      <x:c r="K14" s="10"/>
-      <x:c r="L14" s="7"/>
+      <x:c r="K14" s="7"/>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="8"/>
@@ -530,8 +513,7 @@
       <x:c r="H15" s="8"/>
       <x:c r="I15" s="7"/>
       <x:c r="J15" s="7"/>
-      <x:c r="K15" s="10"/>
-      <x:c r="L15" s="7"/>
+      <x:c r="K15" s="7"/>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
       <x:c r="A16" s="8"/>
@@ -544,8 +526,7 @@
       <x:c r="H16" s="8"/>
       <x:c r="I16" s="7"/>
       <x:c r="J16" s="7"/>
-      <x:c r="K16" s="10"/>
-      <x:c r="L16" s="7"/>
+      <x:c r="K16" s="7"/>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="8"/>
@@ -558,8 +539,7 @@
       <x:c r="H17" s="8"/>
       <x:c r="I17" s="7"/>
       <x:c r="J17" s="7"/>
-      <x:c r="K17" s="10"/>
-      <x:c r="L17" s="7"/>
+      <x:c r="K17" s="7"/>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="8"/>
@@ -572,8 +552,7 @@
       <x:c r="H18" s="8"/>
       <x:c r="I18" s="7"/>
       <x:c r="J18" s="7"/>
-      <x:c r="K18" s="10"/>
-      <x:c r="L18" s="7"/>
+      <x:c r="K18" s="7"/>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="8"/>
@@ -586,8 +565,7 @@
       <x:c r="H19" s="8"/>
       <x:c r="I19" s="7"/>
       <x:c r="J19" s="7"/>
-      <x:c r="K19" s="10"/>
-      <x:c r="L19" s="7"/>
+      <x:c r="K19" s="7"/>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
       <x:c r="A20" s="8"/>
@@ -600,8 +578,7 @@
       <x:c r="H20" s="8"/>
       <x:c r="I20" s="7"/>
       <x:c r="J20" s="7"/>
-      <x:c r="K20" s="10"/>
-      <x:c r="L20" s="7"/>
+      <x:c r="K20" s="7"/>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="8"/>
@@ -614,8 +591,7 @@
       <x:c r="H21" s="8"/>
       <x:c r="I21" s="7"/>
       <x:c r="J21" s="7"/>
-      <x:c r="K21" s="10"/>
-      <x:c r="L21" s="7"/>
+      <x:c r="K21" s="7"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="9"/>
@@ -624,7 +600,6 @@
       <x:c r="E22" s="9"/>
       <x:c r="G22" s="9"/>
       <x:c r="H22" s="9"/>
-      <x:c r="K22" s="11"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="9"/>
@@ -633,7 +608,6 @@
       <x:c r="E23" s="9"/>
       <x:c r="G23" s="9"/>
       <x:c r="H23" s="9"/>
-      <x:c r="K23" s="11"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="9"/>
@@ -642,7 +616,6 @@
       <x:c r="E24" s="9"/>
       <x:c r="G24" s="9"/>
       <x:c r="H24" s="9"/>
-      <x:c r="K24" s="11"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="9"/>
@@ -651,7 +624,6 @@
       <x:c r="E25" s="9"/>
       <x:c r="G25" s="9"/>
       <x:c r="H25" s="9"/>
-      <x:c r="K25" s="11"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="9"/>
@@ -660,7 +632,6 @@
       <x:c r="E26" s="9"/>
       <x:c r="G26" s="9"/>
       <x:c r="H26" s="9"/>
-      <x:c r="K26" s="11"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="9"/>
@@ -669,7 +640,6 @@
       <x:c r="E27" s="9"/>
       <x:c r="G27" s="9"/>
       <x:c r="H27" s="9"/>
-      <x:c r="K27" s="11"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="9"/>
@@ -678,7 +648,6 @@
       <x:c r="E28" s="9"/>
       <x:c r="G28" s="9"/>
       <x:c r="H28" s="9"/>
-      <x:c r="K28" s="11"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="9"/>
@@ -687,7 +656,6 @@
       <x:c r="E29" s="9"/>
       <x:c r="G29" s="9"/>
       <x:c r="H29" s="9"/>
-      <x:c r="K29" s="11"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="9"/>
@@ -696,7 +664,6 @@
       <x:c r="E30" s="9"/>
       <x:c r="G30" s="9"/>
       <x:c r="H30" s="9"/>
-      <x:c r="K30" s="11"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="9"/>
@@ -705,7 +672,6 @@
       <x:c r="E31" s="9"/>
       <x:c r="G31" s="9"/>
       <x:c r="H31" s="9"/>
-      <x:c r="K31" s="11"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="9"/>
@@ -714,7 +680,6 @@
       <x:c r="E32" s="9"/>
       <x:c r="G32" s="9"/>
       <x:c r="H32" s="9"/>
-      <x:c r="K32" s="11"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="9"/>
@@ -723,7 +688,6 @@
       <x:c r="E33" s="9"/>
       <x:c r="G33" s="9"/>
       <x:c r="H33" s="9"/>
-      <x:c r="K33" s="11"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="9"/>
@@ -732,7 +696,6 @@
       <x:c r="E34" s="9"/>
       <x:c r="G34" s="9"/>
       <x:c r="H34" s="9"/>
-      <x:c r="K34" s="11"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="9"/>
@@ -741,7 +704,6 @@
       <x:c r="E35" s="9"/>
       <x:c r="G35" s="9"/>
       <x:c r="H35" s="9"/>
-      <x:c r="K35" s="11"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="9"/>
@@ -750,7 +712,6 @@
       <x:c r="E36" s="9"/>
       <x:c r="G36" s="9"/>
       <x:c r="H36" s="9"/>
-      <x:c r="K36" s="11"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="9"/>
@@ -759,7 +720,6 @@
       <x:c r="E37" s="9"/>
       <x:c r="G37" s="9"/>
       <x:c r="H37" s="9"/>
-      <x:c r="K37" s="11"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="9"/>
@@ -768,7 +728,6 @@
       <x:c r="E38" s="9"/>
       <x:c r="G38" s="9"/>
       <x:c r="H38" s="9"/>
-      <x:c r="K38" s="11"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="9"/>
@@ -777,7 +736,6 @@
       <x:c r="E39" s="9"/>
       <x:c r="G39" s="9"/>
       <x:c r="H39" s="9"/>
-      <x:c r="K39" s="11"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="9"/>
@@ -786,7 +744,6 @@
       <x:c r="E40" s="9"/>
       <x:c r="G40" s="9"/>
       <x:c r="H40" s="9"/>
-      <x:c r="K40" s="11"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="9"/>
@@ -795,7 +752,6 @@
       <x:c r="E41" s="9"/>
       <x:c r="G41" s="9"/>
       <x:c r="H41" s="9"/>
-      <x:c r="K41" s="11"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="9"/>
@@ -804,7 +760,6 @@
       <x:c r="E42" s="9"/>
       <x:c r="G42" s="9"/>
       <x:c r="H42" s="9"/>
-      <x:c r="K42" s="11"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="9"/>
@@ -813,7 +768,6 @@
       <x:c r="E43" s="9"/>
       <x:c r="G43" s="9"/>
       <x:c r="H43" s="9"/>
-      <x:c r="K43" s="11"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="9"/>
@@ -822,7 +776,6 @@
       <x:c r="E44" s="9"/>
       <x:c r="G44" s="9"/>
       <x:c r="H44" s="9"/>
-      <x:c r="K44" s="11"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="9"/>
@@ -831,7 +784,6 @@
       <x:c r="E45" s="9"/>
       <x:c r="G45" s="9"/>
       <x:c r="H45" s="9"/>
-      <x:c r="K45" s="11"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="9"/>
@@ -840,7 +792,6 @@
       <x:c r="E46" s="9"/>
       <x:c r="G46" s="9"/>
       <x:c r="H46" s="9"/>
-      <x:c r="K46" s="11"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="9"/>
@@ -849,7 +800,6 @@
       <x:c r="E47" s="9"/>
       <x:c r="G47" s="9"/>
       <x:c r="H47" s="9"/>
-      <x:c r="K47" s="11"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="9"/>
@@ -858,7 +808,6 @@
       <x:c r="E48" s="9"/>
       <x:c r="G48" s="9"/>
       <x:c r="H48" s="9"/>
-      <x:c r="K48" s="11"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="9"/>
@@ -867,7 +816,6 @@
       <x:c r="E49" s="9"/>
       <x:c r="G49" s="9"/>
       <x:c r="H49" s="9"/>
-      <x:c r="K49" s="11"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="9"/>
@@ -876,7 +824,6 @@
       <x:c r="E50" s="9"/>
       <x:c r="G50" s="9"/>
       <x:c r="H50" s="9"/>
-      <x:c r="K50" s="11"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="9"/>
@@ -885,7 +832,6 @@
       <x:c r="E51" s="9"/>
       <x:c r="G51" s="9"/>
       <x:c r="H51" s="9"/>
-      <x:c r="K51" s="11"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="9"/>
@@ -894,7 +840,6 @@
       <x:c r="E52" s="9"/>
       <x:c r="G52" s="9"/>
       <x:c r="H52" s="9"/>
-      <x:c r="K52" s="11"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="9"/>
@@ -903,7 +848,6 @@
       <x:c r="E53" s="9"/>
       <x:c r="G53" s="9"/>
       <x:c r="H53" s="9"/>
-      <x:c r="K53" s="11"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="9"/>
@@ -912,7 +856,6 @@
       <x:c r="E54" s="9"/>
       <x:c r="G54" s="9"/>
       <x:c r="H54" s="9"/>
-      <x:c r="K54" s="11"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="9"/>
@@ -921,7 +864,6 @@
       <x:c r="E55" s="9"/>
       <x:c r="G55" s="9"/>
       <x:c r="H55" s="9"/>
-      <x:c r="K55" s="11"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="9"/>
@@ -930,7 +872,6 @@
       <x:c r="E56" s="9"/>
       <x:c r="G56" s="9"/>
       <x:c r="H56" s="9"/>
-      <x:c r="K56" s="11"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="9"/>
@@ -939,7 +880,6 @@
       <x:c r="E57" s="9"/>
       <x:c r="G57" s="9"/>
       <x:c r="H57" s="9"/>
-      <x:c r="K57" s="11"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="9"/>
@@ -948,7 +888,6 @@
       <x:c r="E58" s="9"/>
       <x:c r="G58" s="9"/>
       <x:c r="H58" s="9"/>
-      <x:c r="K58" s="11"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="9"/>
@@ -957,7 +896,6 @@
       <x:c r="E59" s="9"/>
       <x:c r="G59" s="9"/>
       <x:c r="H59" s="9"/>
-      <x:c r="K59" s="11"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="9"/>
@@ -966,7 +904,6 @@
       <x:c r="E60" s="9"/>
       <x:c r="G60" s="9"/>
       <x:c r="H60" s="9"/>
-      <x:c r="K60" s="11"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="9"/>
@@ -975,7 +912,6 @@
       <x:c r="E61" s="9"/>
       <x:c r="G61" s="9"/>
       <x:c r="H61" s="9"/>
-      <x:c r="K61" s="11"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="9"/>
@@ -984,7 +920,6 @@
       <x:c r="E62" s="9"/>
       <x:c r="G62" s="9"/>
       <x:c r="H62" s="9"/>
-      <x:c r="K62" s="11"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="9"/>
@@ -993,7 +928,6 @@
       <x:c r="E63" s="9"/>
       <x:c r="G63" s="9"/>
       <x:c r="H63" s="9"/>
-      <x:c r="K63" s="11"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="9"/>
@@ -1002,7 +936,6 @@
       <x:c r="E64" s="9"/>
       <x:c r="G64" s="9"/>
       <x:c r="H64" s="9"/>
-      <x:c r="K64" s="11"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="9"/>
@@ -1011,7 +944,6 @@
       <x:c r="E65" s="9"/>
       <x:c r="G65" s="9"/>
       <x:c r="H65" s="9"/>
-      <x:c r="K65" s="11"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="9"/>
@@ -1020,7 +952,6 @@
       <x:c r="E66" s="9"/>
       <x:c r="G66" s="9"/>
       <x:c r="H66" s="9"/>
-      <x:c r="K66" s="11"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="9"/>
@@ -1029,7 +960,6 @@
       <x:c r="E67" s="9"/>
       <x:c r="G67" s="9"/>
       <x:c r="H67" s="9"/>
-      <x:c r="K67" s="11"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="9"/>
@@ -1038,7 +968,6 @@
       <x:c r="E68" s="9"/>
       <x:c r="G68" s="9"/>
       <x:c r="H68" s="9"/>
-      <x:c r="K68" s="11"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="9"/>
@@ -1047,7 +976,6 @@
       <x:c r="E69" s="9"/>
       <x:c r="G69" s="9"/>
       <x:c r="H69" s="9"/>
-      <x:c r="K69" s="11"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="9"/>
@@ -1056,7 +984,6 @@
       <x:c r="E70" s="9"/>
       <x:c r="G70" s="9"/>
       <x:c r="H70" s="9"/>
-      <x:c r="K70" s="11"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="9"/>
@@ -1065,7 +992,6 @@
       <x:c r="E71" s="9"/>
       <x:c r="G71" s="9"/>
       <x:c r="H71" s="9"/>
-      <x:c r="K71" s="11"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="9"/>
@@ -1074,7 +1000,6 @@
       <x:c r="E72" s="9"/>
       <x:c r="G72" s="9"/>
       <x:c r="H72" s="9"/>
-      <x:c r="K72" s="11"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="9"/>
@@ -1083,7 +1008,6 @@
       <x:c r="E73" s="9"/>
       <x:c r="G73" s="9"/>
       <x:c r="H73" s="9"/>
-      <x:c r="K73" s="11"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="9"/>
@@ -1092,7 +1016,6 @@
       <x:c r="E74" s="9"/>
       <x:c r="G74" s="9"/>
       <x:c r="H74" s="9"/>
-      <x:c r="K74" s="11"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="9"/>
@@ -1101,7 +1024,6 @@
       <x:c r="E75" s="9"/>
       <x:c r="G75" s="9"/>
       <x:c r="H75" s="9"/>
-      <x:c r="K75" s="11"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="9"/>
@@ -1110,7 +1032,6 @@
       <x:c r="E76" s="9"/>
       <x:c r="G76" s="9"/>
       <x:c r="H76" s="9"/>
-      <x:c r="K76" s="11"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="9"/>
@@ -1119,7 +1040,6 @@
       <x:c r="E77" s="9"/>
       <x:c r="G77" s="9"/>
       <x:c r="H77" s="9"/>
-      <x:c r="K77" s="11"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="9"/>
@@ -1128,7 +1048,6 @@
       <x:c r="E78" s="9"/>
       <x:c r="G78" s="9"/>
       <x:c r="H78" s="9"/>
-      <x:c r="K78" s="11"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="9"/>
@@ -1137,7 +1056,6 @@
       <x:c r="E79" s="9"/>
       <x:c r="G79" s="9"/>
       <x:c r="H79" s="9"/>
-      <x:c r="K79" s="11"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="9"/>
@@ -1146,7 +1064,6 @@
       <x:c r="E80" s="9"/>
       <x:c r="G80" s="9"/>
       <x:c r="H80" s="9"/>
-      <x:c r="K80" s="11"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="9"/>
@@ -1155,7 +1072,6 @@
       <x:c r="E81" s="9"/>
       <x:c r="G81" s="9"/>
       <x:c r="H81" s="9"/>
-      <x:c r="K81" s="11"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="9"/>
@@ -1164,7 +1080,6 @@
       <x:c r="E82" s="9"/>
       <x:c r="G82" s="9"/>
       <x:c r="H82" s="9"/>
-      <x:c r="K82" s="11"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="9"/>
@@ -1173,7 +1088,6 @@
       <x:c r="E83" s="9"/>
       <x:c r="G83" s="9"/>
       <x:c r="H83" s="9"/>
-      <x:c r="K83" s="11"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="9"/>
@@ -1182,7 +1096,6 @@
       <x:c r="E84" s="9"/>
       <x:c r="G84" s="9"/>
       <x:c r="H84" s="9"/>
-      <x:c r="K84" s="11"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="9"/>
@@ -1191,7 +1104,6 @@
       <x:c r="E85" s="9"/>
       <x:c r="G85" s="9"/>
       <x:c r="H85" s="9"/>
-      <x:c r="K85" s="11"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="9"/>
@@ -1200,7 +1112,6 @@
       <x:c r="E86" s="9"/>
       <x:c r="G86" s="9"/>
       <x:c r="H86" s="9"/>
-      <x:c r="K86" s="11"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="9"/>
@@ -1209,7 +1120,6 @@
       <x:c r="E87" s="9"/>
       <x:c r="G87" s="9"/>
       <x:c r="H87" s="9"/>
-      <x:c r="K87" s="11"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="9"/>
@@ -1218,7 +1128,6 @@
       <x:c r="E88" s="9"/>
       <x:c r="G88" s="9"/>
       <x:c r="H88" s="9"/>
-      <x:c r="K88" s="11"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="9"/>
@@ -1227,7 +1136,6 @@
       <x:c r="E89" s="9"/>
       <x:c r="G89" s="9"/>
       <x:c r="H89" s="9"/>
-      <x:c r="K89" s="11"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="9"/>
@@ -1236,7 +1144,6 @@
       <x:c r="E90" s="9"/>
       <x:c r="G90" s="9"/>
       <x:c r="H90" s="9"/>
-      <x:c r="K90" s="11"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="9"/>
@@ -1245,7 +1152,6 @@
       <x:c r="E91" s="9"/>
       <x:c r="G91" s="9"/>
       <x:c r="H91" s="9"/>
-      <x:c r="K91" s="11"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="9"/>
@@ -1254,7 +1160,6 @@
       <x:c r="E92" s="9"/>
       <x:c r="G92" s="9"/>
       <x:c r="H92" s="9"/>
-      <x:c r="K92" s="11"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="9"/>
@@ -1263,7 +1168,6 @@
       <x:c r="E93" s="9"/>
       <x:c r="G93" s="9"/>
       <x:c r="H93" s="9"/>
-      <x:c r="K93" s="11"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="9"/>
@@ -1272,7 +1176,6 @@
       <x:c r="E94" s="9"/>
       <x:c r="G94" s="9"/>
       <x:c r="H94" s="9"/>
-      <x:c r="K94" s="11"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="9"/>
@@ -1281,7 +1184,6 @@
       <x:c r="E95" s="9"/>
       <x:c r="G95" s="9"/>
       <x:c r="H95" s="9"/>
-      <x:c r="K95" s="11"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="9"/>
@@ -1290,7 +1192,6 @@
       <x:c r="E96" s="9"/>
       <x:c r="G96" s="9"/>
       <x:c r="H96" s="9"/>
-      <x:c r="K96" s="11"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="9"/>
@@ -1299,7 +1200,6 @@
       <x:c r="E97" s="9"/>
       <x:c r="G97" s="9"/>
       <x:c r="H97" s="9"/>
-      <x:c r="K97" s="11"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="9"/>
@@ -1308,7 +1208,6 @@
       <x:c r="E98" s="9"/>
       <x:c r="G98" s="9"/>
       <x:c r="H98" s="9"/>
-      <x:c r="K98" s="11"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="9"/>
@@ -1317,7 +1216,6 @@
       <x:c r="E99" s="9"/>
       <x:c r="G99" s="9"/>
       <x:c r="H99" s="9"/>
-      <x:c r="K99" s="11"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="9"/>
@@ -1326,7 +1224,6 @@
       <x:c r="E100" s="9"/>
       <x:c r="G100" s="9"/>
       <x:c r="H100" s="9"/>
-      <x:c r="K100" s="11"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="9"/>
@@ -1335,7 +1232,6 @@
       <x:c r="E101" s="9"/>
       <x:c r="G101" s="9"/>
       <x:c r="H101" s="9"/>
-      <x:c r="K101" s="11"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="9"/>
@@ -1344,7 +1240,6 @@
       <x:c r="E102" s="9"/>
       <x:c r="G102" s="9"/>
       <x:c r="H102" s="9"/>
-      <x:c r="K102" s="11"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="9"/>
@@ -1353,7 +1248,6 @@
       <x:c r="E103" s="9"/>
       <x:c r="G103" s="9"/>
       <x:c r="H103" s="9"/>
-      <x:c r="K103" s="11"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="9"/>
@@ -1362,7 +1256,6 @@
       <x:c r="E104" s="9"/>
       <x:c r="G104" s="9"/>
       <x:c r="H104" s="9"/>
-      <x:c r="K104" s="11"/>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="9"/>
@@ -1371,7 +1264,6 @@
       <x:c r="E105" s="9"/>
       <x:c r="G105" s="9"/>
       <x:c r="H105" s="9"/>
-      <x:c r="K105" s="11"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="9"/>
@@ -1380,7 +1272,6 @@
       <x:c r="E106" s="9"/>
       <x:c r="G106" s="9"/>
       <x:c r="H106" s="9"/>
-      <x:c r="K106" s="11"/>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="9"/>
@@ -1389,7 +1280,6 @@
       <x:c r="E107" s="9"/>
       <x:c r="G107" s="9"/>
       <x:c r="H107" s="9"/>
-      <x:c r="K107" s="11"/>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="9"/>
@@ -1398,7 +1288,6 @@
       <x:c r="E108" s="9"/>
       <x:c r="G108" s="9"/>
       <x:c r="H108" s="9"/>
-      <x:c r="K108" s="11"/>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="9"/>
@@ -1407,7 +1296,6 @@
       <x:c r="E109" s="9"/>
       <x:c r="G109" s="9"/>
       <x:c r="H109" s="9"/>
-      <x:c r="K109" s="11"/>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="9"/>
@@ -1416,7 +1304,6 @@
       <x:c r="E110" s="9"/>
       <x:c r="G110" s="9"/>
       <x:c r="H110" s="9"/>
-      <x:c r="K110" s="11"/>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="9"/>
@@ -1425,7 +1312,6 @@
       <x:c r="E111" s="9"/>
       <x:c r="G111" s="9"/>
       <x:c r="H111" s="9"/>
-      <x:c r="K111" s="11"/>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="9"/>
@@ -1434,7 +1320,6 @@
       <x:c r="E112" s="9"/>
       <x:c r="G112" s="9"/>
       <x:c r="H112" s="9"/>
-      <x:c r="K112" s="11"/>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="9"/>
@@ -1443,7 +1328,6 @@
       <x:c r="E113" s="9"/>
       <x:c r="G113" s="9"/>
       <x:c r="H113" s="9"/>
-      <x:c r="K113" s="11"/>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="9"/>
@@ -1452,7 +1336,6 @@
       <x:c r="E114" s="9"/>
       <x:c r="G114" s="9"/>
       <x:c r="H114" s="9"/>
-      <x:c r="K114" s="11"/>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="9"/>
@@ -1461,7 +1344,6 @@
       <x:c r="E115" s="9"/>
       <x:c r="G115" s="9"/>
       <x:c r="H115" s="9"/>
-      <x:c r="K115" s="11"/>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="9"/>
@@ -1470,7 +1352,6 @@
       <x:c r="E116" s="9"/>
       <x:c r="G116" s="9"/>
       <x:c r="H116" s="9"/>
-      <x:c r="K116" s="11"/>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="9"/>
@@ -1479,7 +1360,6 @@
       <x:c r="E117" s="9"/>
       <x:c r="G117" s="9"/>
       <x:c r="H117" s="9"/>
-      <x:c r="K117" s="11"/>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="9"/>
@@ -1488,7 +1368,6 @@
       <x:c r="E118" s="9"/>
       <x:c r="G118" s="9"/>
       <x:c r="H118" s="9"/>
-      <x:c r="K118" s="11"/>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="9"/>
@@ -1497,7 +1376,6 @@
       <x:c r="E119" s="9"/>
       <x:c r="G119" s="9"/>
       <x:c r="H119" s="9"/>
-      <x:c r="K119" s="11"/>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="9"/>
@@ -1506,7 +1384,6 @@
       <x:c r="E120" s="9"/>
       <x:c r="G120" s="9"/>
       <x:c r="H120" s="9"/>
-      <x:c r="K120" s="11"/>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="9"/>
@@ -1515,7 +1392,6 @@
       <x:c r="E121" s="9"/>
       <x:c r="G121" s="9"/>
       <x:c r="H121" s="9"/>
-      <x:c r="K121" s="11"/>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="9"/>
@@ -1524,7 +1400,6 @@
       <x:c r="E122" s="9"/>
       <x:c r="G122" s="9"/>
       <x:c r="H122" s="9"/>
-      <x:c r="K122" s="11"/>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="9"/>
@@ -1533,7 +1408,6 @@
       <x:c r="E123" s="9"/>
       <x:c r="G123" s="9"/>
       <x:c r="H123" s="9"/>
-      <x:c r="K123" s="11"/>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="9"/>
@@ -1542,7 +1416,6 @@
       <x:c r="E124" s="9"/>
       <x:c r="G124" s="9"/>
       <x:c r="H124" s="9"/>
-      <x:c r="K124" s="11"/>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="9"/>
@@ -1551,7 +1424,6 @@
       <x:c r="E125" s="9"/>
       <x:c r="G125" s="9"/>
       <x:c r="H125" s="9"/>
-      <x:c r="K125" s="11"/>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="9"/>
@@ -1560,7 +1432,6 @@
       <x:c r="E126" s="9"/>
       <x:c r="G126" s="9"/>
       <x:c r="H126" s="9"/>
-      <x:c r="K126" s="11"/>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="9"/>
@@ -1569,7 +1440,6 @@
       <x:c r="E127" s="9"/>
       <x:c r="G127" s="9"/>
       <x:c r="H127" s="9"/>
-      <x:c r="K127" s="11"/>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="9"/>
@@ -1578,7 +1448,6 @@
       <x:c r="E128" s="9"/>
       <x:c r="G128" s="9"/>
       <x:c r="H128" s="9"/>
-      <x:c r="K128" s="11"/>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="9"/>
@@ -1587,7 +1456,6 @@
       <x:c r="E129" s="9"/>
       <x:c r="G129" s="9"/>
       <x:c r="H129" s="9"/>
-      <x:c r="K129" s="11"/>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="9"/>
@@ -1596,7 +1464,6 @@
       <x:c r="E130" s="9"/>
       <x:c r="G130" s="9"/>
       <x:c r="H130" s="9"/>
-      <x:c r="K130" s="11"/>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="9"/>
@@ -1605,7 +1472,6 @@
       <x:c r="E131" s="9"/>
       <x:c r="G131" s="9"/>
       <x:c r="H131" s="9"/>
-      <x:c r="K131" s="11"/>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="9"/>
@@ -1614,7 +1480,6 @@
       <x:c r="E132" s="9"/>
       <x:c r="G132" s="9"/>
       <x:c r="H132" s="9"/>
-      <x:c r="K132" s="11"/>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="9"/>
@@ -1623,7 +1488,6 @@
       <x:c r="E133" s="9"/>
       <x:c r="G133" s="9"/>
       <x:c r="H133" s="9"/>
-      <x:c r="K133" s="11"/>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="9"/>
@@ -1632,7 +1496,6 @@
       <x:c r="E134" s="9"/>
       <x:c r="G134" s="9"/>
       <x:c r="H134" s="9"/>
-      <x:c r="K134" s="11"/>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="9"/>
@@ -1641,7 +1504,6 @@
       <x:c r="E135" s="9"/>
       <x:c r="G135" s="9"/>
       <x:c r="H135" s="9"/>
-      <x:c r="K135" s="11"/>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="9"/>
@@ -1650,7 +1512,6 @@
       <x:c r="E136" s="9"/>
       <x:c r="G136" s="9"/>
       <x:c r="H136" s="9"/>
-      <x:c r="K136" s="11"/>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="9"/>
@@ -1659,7 +1520,6 @@
       <x:c r="E137" s="9"/>
       <x:c r="G137" s="9"/>
       <x:c r="H137" s="9"/>
-      <x:c r="K137" s="11"/>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="9"/>
@@ -1668,7 +1528,6 @@
       <x:c r="E138" s="9"/>
       <x:c r="G138" s="9"/>
       <x:c r="H138" s="9"/>
-      <x:c r="K138" s="11"/>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="9"/>
@@ -1677,7 +1536,6 @@
       <x:c r="E139" s="9"/>
       <x:c r="G139" s="9"/>
       <x:c r="H139" s="9"/>
-      <x:c r="K139" s="11"/>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="9"/>
@@ -1686,7 +1544,6 @@
       <x:c r="E140" s="9"/>
       <x:c r="G140" s="9"/>
       <x:c r="H140" s="9"/>
-      <x:c r="K140" s="11"/>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="9"/>
@@ -1695,7 +1552,6 @@
       <x:c r="E141" s="9"/>
       <x:c r="G141" s="9"/>
       <x:c r="H141" s="9"/>
-      <x:c r="K141" s="11"/>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="9"/>
@@ -1704,7 +1560,6 @@
       <x:c r="E142" s="9"/>
       <x:c r="G142" s="9"/>
       <x:c r="H142" s="9"/>
-      <x:c r="K142" s="11"/>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="9"/>
@@ -1713,7 +1568,6 @@
       <x:c r="E143" s="9"/>
       <x:c r="G143" s="9"/>
       <x:c r="H143" s="9"/>
-      <x:c r="K143" s="11"/>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="9"/>
@@ -1722,7 +1576,6 @@
       <x:c r="E144" s="9"/>
       <x:c r="G144" s="9"/>
       <x:c r="H144" s="9"/>
-      <x:c r="K144" s="11"/>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="9"/>
@@ -1731,7 +1584,6 @@
       <x:c r="E145" s="9"/>
       <x:c r="G145" s="9"/>
       <x:c r="H145" s="9"/>
-      <x:c r="K145" s="11"/>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="9"/>
@@ -1740,7 +1592,6 @@
       <x:c r="E146" s="9"/>
       <x:c r="G146" s="9"/>
       <x:c r="H146" s="9"/>
-      <x:c r="K146" s="11"/>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="9"/>
@@ -1749,7 +1600,6 @@
       <x:c r="E147" s="9"/>
       <x:c r="G147" s="9"/>
       <x:c r="H147" s="9"/>
-      <x:c r="K147" s="11"/>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="9"/>
@@ -1758,7 +1608,6 @@
       <x:c r="E148" s="9"/>
       <x:c r="G148" s="9"/>
       <x:c r="H148" s="9"/>
-      <x:c r="K148" s="11"/>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="9"/>
@@ -1767,7 +1616,6 @@
       <x:c r="E149" s="9"/>
       <x:c r="G149" s="9"/>
       <x:c r="H149" s="9"/>
-      <x:c r="K149" s="11"/>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="9"/>
@@ -1776,7 +1624,6 @@
       <x:c r="E150" s="9"/>
       <x:c r="G150" s="9"/>
       <x:c r="H150" s="9"/>
-      <x:c r="K150" s="11"/>
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="9"/>
@@ -1785,7 +1632,6 @@
       <x:c r="E151" s="9"/>
       <x:c r="G151" s="9"/>
       <x:c r="H151" s="9"/>
-      <x:c r="K151" s="11"/>
     </x:row>
     <x:row r="152">
       <x:c r="A152" s="9"/>
@@ -1794,7 +1640,6 @@
       <x:c r="E152" s="9"/>
       <x:c r="G152" s="9"/>
       <x:c r="H152" s="9"/>
-      <x:c r="K152" s="11"/>
     </x:row>
     <x:row r="153">
       <x:c r="A153" s="9"/>
@@ -1803,7 +1648,6 @@
       <x:c r="E153" s="9"/>
       <x:c r="G153" s="9"/>
       <x:c r="H153" s="9"/>
-      <x:c r="K153" s="11"/>
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="9"/>
@@ -1812,7 +1656,6 @@
       <x:c r="E154" s="9"/>
       <x:c r="G154" s="9"/>
       <x:c r="H154" s="9"/>
-      <x:c r="K154" s="11"/>
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="9"/>
@@ -1821,7 +1664,6 @@
       <x:c r="E155" s="9"/>
       <x:c r="G155" s="9"/>
       <x:c r="H155" s="9"/>
-      <x:c r="K155" s="11"/>
     </x:row>
     <x:row r="156">
       <x:c r="A156" s="9"/>
@@ -1830,7 +1672,6 @@
       <x:c r="E156" s="9"/>
       <x:c r="G156" s="9"/>
       <x:c r="H156" s="9"/>
-      <x:c r="K156" s="11"/>
     </x:row>
     <x:row r="157">
       <x:c r="A157" s="9"/>
@@ -1839,7 +1680,6 @@
       <x:c r="E157" s="9"/>
       <x:c r="G157" s="9"/>
       <x:c r="H157" s="9"/>
-      <x:c r="K157" s="11"/>
     </x:row>
     <x:row r="158">
       <x:c r="A158" s="9"/>
@@ -1848,7 +1688,6 @@
       <x:c r="E158" s="9"/>
       <x:c r="G158" s="9"/>
       <x:c r="H158" s="9"/>
-      <x:c r="K158" s="11"/>
     </x:row>
     <x:row r="159">
       <x:c r="A159" s="9"/>
@@ -1857,7 +1696,6 @@
       <x:c r="E159" s="9"/>
       <x:c r="G159" s="9"/>
       <x:c r="H159" s="9"/>
-      <x:c r="K159" s="11"/>
     </x:row>
     <x:row r="160">
       <x:c r="A160" s="9"/>
@@ -1866,7 +1704,6 @@
       <x:c r="E160" s="9"/>
       <x:c r="G160" s="9"/>
       <x:c r="H160" s="9"/>
-      <x:c r="K160" s="11"/>
     </x:row>
     <x:row r="161">
       <x:c r="A161" s="9"/>
@@ -1875,7 +1712,6 @@
       <x:c r="E161" s="9"/>
       <x:c r="G161" s="9"/>
       <x:c r="H161" s="9"/>
-      <x:c r="K161" s="11"/>
     </x:row>
     <x:row r="162">
       <x:c r="A162" s="9"/>
@@ -1884,7 +1720,6 @@
       <x:c r="E162" s="9"/>
       <x:c r="G162" s="9"/>
       <x:c r="H162" s="9"/>
-      <x:c r="K162" s="11"/>
     </x:row>
     <x:row r="163">
       <x:c r="A163" s="9"/>
@@ -1893,7 +1728,6 @@
       <x:c r="E163" s="9"/>
       <x:c r="G163" s="9"/>
       <x:c r="H163" s="9"/>
-      <x:c r="K163" s="11"/>
     </x:row>
     <x:row r="164">
       <x:c r="A164" s="9"/>
@@ -1902,7 +1736,6 @@
       <x:c r="E164" s="9"/>
       <x:c r="G164" s="9"/>
       <x:c r="H164" s="9"/>
-      <x:c r="K164" s="11"/>
     </x:row>
     <x:row r="165">
       <x:c r="A165" s="9"/>
@@ -1911,7 +1744,6 @@
       <x:c r="E165" s="9"/>
       <x:c r="G165" s="9"/>
       <x:c r="H165" s="9"/>
-      <x:c r="K165" s="11"/>
     </x:row>
     <x:row r="166">
       <x:c r="A166" s="9"/>
@@ -1920,7 +1752,6 @@
       <x:c r="E166" s="9"/>
       <x:c r="G166" s="9"/>
       <x:c r="H166" s="9"/>
-      <x:c r="K166" s="11"/>
     </x:row>
     <x:row r="167">
       <x:c r="A167" s="9"/>
@@ -1929,7 +1760,6 @@
       <x:c r="E167" s="9"/>
       <x:c r="G167" s="9"/>
       <x:c r="H167" s="9"/>
-      <x:c r="K167" s="11"/>
     </x:row>
     <x:row r="168">
       <x:c r="A168" s="9"/>
@@ -1938,7 +1768,6 @@
       <x:c r="E168" s="9"/>
       <x:c r="G168" s="9"/>
       <x:c r="H168" s="9"/>
-      <x:c r="K168" s="11"/>
     </x:row>
     <x:row r="169">
       <x:c r="A169" s="9"/>
@@ -1947,7 +1776,6 @@
       <x:c r="E169" s="9"/>
       <x:c r="G169" s="9"/>
       <x:c r="H169" s="9"/>
-      <x:c r="K169" s="11"/>
     </x:row>
     <x:row r="170">
       <x:c r="A170" s="9"/>
@@ -1956,7 +1784,6 @@
       <x:c r="E170" s="9"/>
       <x:c r="G170" s="9"/>
       <x:c r="H170" s="9"/>
-      <x:c r="K170" s="11"/>
     </x:row>
     <x:row r="171">
       <x:c r="A171" s="9"/>
@@ -1965,7 +1792,6 @@
       <x:c r="E171" s="9"/>
       <x:c r="G171" s="9"/>
       <x:c r="H171" s="9"/>
-      <x:c r="K171" s="11"/>
     </x:row>
     <x:row r="172">
       <x:c r="A172" s="9"/>
@@ -1974,7 +1800,6 @@
       <x:c r="E172" s="9"/>
       <x:c r="G172" s="9"/>
       <x:c r="H172" s="9"/>
-      <x:c r="K172" s="11"/>
     </x:row>
     <x:row r="173">
       <x:c r="A173" s="9"/>
@@ -1983,7 +1808,6 @@
       <x:c r="E173" s="9"/>
       <x:c r="G173" s="9"/>
       <x:c r="H173" s="9"/>
-      <x:c r="K173" s="11"/>
     </x:row>
     <x:row r="174">
       <x:c r="A174" s="9"/>
@@ -1992,7 +1816,6 @@
       <x:c r="E174" s="9"/>
       <x:c r="G174" s="9"/>
       <x:c r="H174" s="9"/>
-      <x:c r="K174" s="11"/>
     </x:row>
     <x:row r="175">
       <x:c r="A175" s="9"/>
@@ -2001,7 +1824,6 @@
       <x:c r="E175" s="9"/>
       <x:c r="G175" s="9"/>
       <x:c r="H175" s="9"/>
-      <x:c r="K175" s="11"/>
     </x:row>
     <x:row r="176">
       <x:c r="A176" s="9"/>
@@ -2010,7 +1832,6 @@
       <x:c r="E176" s="9"/>
       <x:c r="G176" s="9"/>
       <x:c r="H176" s="9"/>
-      <x:c r="K176" s="11"/>
     </x:row>
     <x:row r="177">
       <x:c r="A177" s="9"/>
@@ -2019,7 +1840,6 @@
       <x:c r="E177" s="9"/>
       <x:c r="G177" s="9"/>
       <x:c r="H177" s="9"/>
-      <x:c r="K177" s="11"/>
     </x:row>
     <x:row r="178">
       <x:c r="A178" s="9"/>
@@ -2028,7 +1848,6 @@
       <x:c r="E178" s="9"/>
       <x:c r="G178" s="9"/>
       <x:c r="H178" s="9"/>
-      <x:c r="K178" s="11"/>
     </x:row>
     <x:row r="179">
       <x:c r="A179" s="9"/>
@@ -2037,7 +1856,6 @@
       <x:c r="E179" s="9"/>
       <x:c r="G179" s="9"/>
       <x:c r="H179" s="9"/>
-      <x:c r="K179" s="11"/>
     </x:row>
     <x:row r="180">
       <x:c r="A180" s="9"/>
@@ -2046,7 +1864,6 @@
       <x:c r="E180" s="9"/>
       <x:c r="G180" s="9"/>
       <x:c r="H180" s="9"/>
-      <x:c r="K180" s="11"/>
     </x:row>
     <x:row r="181">
       <x:c r="A181" s="9"/>
@@ -2055,7 +1872,6 @@
       <x:c r="E181" s="9"/>
       <x:c r="G181" s="9"/>
       <x:c r="H181" s="9"/>
-      <x:c r="K181" s="11"/>
     </x:row>
     <x:row r="182">
       <x:c r="A182" s="9"/>
@@ -2064,7 +1880,6 @@
       <x:c r="E182" s="9"/>
       <x:c r="G182" s="9"/>
       <x:c r="H182" s="9"/>
-      <x:c r="K182" s="11"/>
     </x:row>
     <x:row r="183">
       <x:c r="A183" s="9"/>
@@ -2073,7 +1888,6 @@
       <x:c r="E183" s="9"/>
       <x:c r="G183" s="9"/>
       <x:c r="H183" s="9"/>
-      <x:c r="K183" s="11"/>
     </x:row>
     <x:row r="184">
       <x:c r="A184" s="9"/>
@@ -2082,7 +1896,6 @@
       <x:c r="E184" s="9"/>
       <x:c r="G184" s="9"/>
       <x:c r="H184" s="9"/>
-      <x:c r="K184" s="11"/>
     </x:row>
     <x:row r="185">
       <x:c r="A185" s="9"/>
@@ -2091,7 +1904,6 @@
       <x:c r="E185" s="9"/>
       <x:c r="G185" s="9"/>
       <x:c r="H185" s="9"/>
-      <x:c r="K185" s="11"/>
     </x:row>
     <x:row r="186">
       <x:c r="A186" s="9"/>
@@ -2100,7 +1912,6 @@
       <x:c r="E186" s="9"/>
       <x:c r="G186" s="9"/>
       <x:c r="H186" s="9"/>
-      <x:c r="K186" s="11"/>
     </x:row>
     <x:row r="187">
       <x:c r="A187" s="9"/>
@@ -2109,7 +1920,6 @@
       <x:c r="E187" s="9"/>
       <x:c r="G187" s="9"/>
       <x:c r="H187" s="9"/>
-      <x:c r="K187" s="11"/>
     </x:row>
     <x:row r="188">
       <x:c r="A188" s="9"/>
@@ -2118,7 +1928,6 @@
       <x:c r="E188" s="9"/>
       <x:c r="G188" s="9"/>
       <x:c r="H188" s="9"/>
-      <x:c r="K188" s="11"/>
     </x:row>
     <x:row r="189">
       <x:c r="A189" s="9"/>
@@ -2127,7 +1936,6 @@
       <x:c r="E189" s="9"/>
       <x:c r="G189" s="9"/>
       <x:c r="H189" s="9"/>
-      <x:c r="K189" s="11"/>
     </x:row>
     <x:row r="190">
       <x:c r="A190" s="9"/>
@@ -2136,7 +1944,6 @@
       <x:c r="E190" s="9"/>
       <x:c r="G190" s="9"/>
       <x:c r="H190" s="9"/>
-      <x:c r="K190" s="11"/>
     </x:row>
     <x:row r="191">
       <x:c r="A191" s="9"/>
@@ -2145,7 +1952,6 @@
       <x:c r="E191" s="9"/>
       <x:c r="G191" s="9"/>
       <x:c r="H191" s="9"/>
-      <x:c r="K191" s="11"/>
     </x:row>
     <x:row r="192">
       <x:c r="A192" s="9"/>
@@ -2154,7 +1960,6 @@
       <x:c r="E192" s="9"/>
       <x:c r="G192" s="9"/>
       <x:c r="H192" s="9"/>
-      <x:c r="K192" s="11"/>
     </x:row>
     <x:row r="193">
       <x:c r="A193" s="9"/>
@@ -2163,7 +1968,6 @@
       <x:c r="E193" s="9"/>
       <x:c r="G193" s="9"/>
       <x:c r="H193" s="9"/>
-      <x:c r="K193" s="11"/>
     </x:row>
     <x:row r="194">
       <x:c r="A194" s="9"/>
@@ -2172,7 +1976,6 @@
       <x:c r="E194" s="9"/>
       <x:c r="G194" s="9"/>
       <x:c r="H194" s="9"/>
-      <x:c r="K194" s="11"/>
     </x:row>
     <x:row r="195">
       <x:c r="A195" s="9"/>
@@ -2181,7 +1984,6 @@
       <x:c r="E195" s="9"/>
       <x:c r="G195" s="9"/>
       <x:c r="H195" s="9"/>
-      <x:c r="K195" s="11"/>
     </x:row>
     <x:row r="196">
       <x:c r="A196" s="9"/>
@@ -2190,7 +1992,6 @@
       <x:c r="E196" s="9"/>
       <x:c r="G196" s="9"/>
       <x:c r="H196" s="9"/>
-      <x:c r="K196" s="11"/>
     </x:row>
     <x:row r="197">
       <x:c r="A197" s="9"/>
@@ -2199,7 +2000,6 @@
       <x:c r="E197" s="9"/>
       <x:c r="G197" s="9"/>
       <x:c r="H197" s="9"/>
-      <x:c r="K197" s="11"/>
     </x:row>
     <x:row r="198">
       <x:c r="A198" s="9"/>
@@ -2208,7 +2008,6 @@
       <x:c r="E198" s="9"/>
       <x:c r="G198" s="9"/>
       <x:c r="H198" s="9"/>
-      <x:c r="K198" s="11"/>
     </x:row>
     <x:row r="199">
       <x:c r="A199" s="9"/>
@@ -2217,7 +2016,6 @@
       <x:c r="E199" s="9"/>
       <x:c r="G199" s="9"/>
       <x:c r="H199" s="9"/>
-      <x:c r="K199" s="11"/>
     </x:row>
     <x:row r="200">
       <x:c r="A200" s="9"/>
@@ -2226,7 +2024,6 @@
       <x:c r="E200" s="9"/>
       <x:c r="G200" s="9"/>
       <x:c r="H200" s="9"/>
-      <x:c r="K200" s="11"/>
     </x:row>
     <x:row r="201">
       <x:c r="A201" s="9"/>
@@ -2235,7 +2032,6 @@
       <x:c r="E201" s="9"/>
       <x:c r="G201" s="9"/>
       <x:c r="H201" s="9"/>
-      <x:c r="K201" s="11"/>
     </x:row>
     <x:row r="202">
       <x:c r="A202" s="9"/>
@@ -2244,7 +2040,6 @@
       <x:c r="E202" s="9"/>
       <x:c r="G202" s="9"/>
       <x:c r="H202" s="9"/>
-      <x:c r="K202" s="11"/>
     </x:row>
     <x:row r="203">
       <x:c r="A203" s="9"/>
@@ -2253,7 +2048,6 @@
       <x:c r="E203" s="9"/>
       <x:c r="G203" s="9"/>
       <x:c r="H203" s="9"/>
-      <x:c r="K203" s="11"/>
     </x:row>
     <x:row r="204">
       <x:c r="A204" s="9"/>
@@ -2262,7 +2056,6 @@
       <x:c r="E204" s="9"/>
       <x:c r="G204" s="9"/>
       <x:c r="H204" s="9"/>
-      <x:c r="K204" s="11"/>
     </x:row>
     <x:row r="205">
       <x:c r="A205" s="9"/>
@@ -2271,7 +2064,6 @@
       <x:c r="E205" s="9"/>
       <x:c r="G205" s="9"/>
       <x:c r="H205" s="9"/>
-      <x:c r="K205" s="11"/>
     </x:row>
     <x:row r="206">
       <x:c r="A206" s="9"/>
@@ -2280,7 +2072,6 @@
       <x:c r="E206" s="9"/>
       <x:c r="G206" s="9"/>
       <x:c r="H206" s="9"/>
-      <x:c r="K206" s="11"/>
     </x:row>
     <x:row r="207">
       <x:c r="A207" s="9"/>
@@ -2289,7 +2080,6 @@
       <x:c r="E207" s="9"/>
       <x:c r="G207" s="9"/>
       <x:c r="H207" s="9"/>
-      <x:c r="K207" s="11"/>
     </x:row>
     <x:row r="208">
       <x:c r="A208" s="9"/>
@@ -2298,7 +2088,6 @@
       <x:c r="E208" s="9"/>
       <x:c r="G208" s="9"/>
       <x:c r="H208" s="9"/>
-      <x:c r="K208" s="11"/>
     </x:row>
     <x:row r="209">
       <x:c r="A209" s="9"/>
@@ -2307,7 +2096,6 @@
       <x:c r="E209" s="9"/>
       <x:c r="G209" s="9"/>
       <x:c r="H209" s="9"/>
-      <x:c r="K209" s="11"/>
     </x:row>
     <x:row r="210">
       <x:c r="A210" s="9"/>
@@ -2316,7 +2104,6 @@
       <x:c r="E210" s="9"/>
       <x:c r="G210" s="9"/>
       <x:c r="H210" s="9"/>
-      <x:c r="K210" s="11"/>
     </x:row>
     <x:row r="211">
       <x:c r="A211" s="9"/>
@@ -2325,7 +2112,6 @@
       <x:c r="E211" s="9"/>
       <x:c r="G211" s="9"/>
       <x:c r="H211" s="9"/>
-      <x:c r="K211" s="11"/>
     </x:row>
     <x:row r="212">
       <x:c r="A212" s="9"/>
@@ -2334,7 +2120,6 @@
       <x:c r="E212" s="9"/>
       <x:c r="G212" s="9"/>
       <x:c r="H212" s="9"/>
-      <x:c r="K212" s="11"/>
     </x:row>
     <x:row r="213">
       <x:c r="A213" s="9"/>
@@ -2343,7 +2128,6 @@
       <x:c r="E213" s="9"/>
       <x:c r="G213" s="9"/>
       <x:c r="H213" s="9"/>
-      <x:c r="K213" s="11"/>
     </x:row>
     <x:row r="214">
       <x:c r="A214" s="9"/>
@@ -2352,7 +2136,6 @@
       <x:c r="E214" s="9"/>
       <x:c r="G214" s="9"/>
       <x:c r="H214" s="9"/>
-      <x:c r="K214" s="11"/>
     </x:row>
     <x:row r="215">
       <x:c r="A215" s="9"/>
@@ -2361,7 +2144,6 @@
       <x:c r="E215" s="9"/>
       <x:c r="G215" s="9"/>
       <x:c r="H215" s="9"/>
-      <x:c r="K215" s="11"/>
     </x:row>
     <x:row r="216">
       <x:c r="A216" s="9"/>
@@ -2370,7 +2152,6 @@
       <x:c r="E216" s="9"/>
       <x:c r="G216" s="9"/>
       <x:c r="H216" s="9"/>
-      <x:c r="K216" s="11"/>
     </x:row>
     <x:row r="217">
       <x:c r="A217" s="9"/>
@@ -2379,7 +2160,6 @@
       <x:c r="E217" s="9"/>
       <x:c r="G217" s="9"/>
       <x:c r="H217" s="9"/>
-      <x:c r="K217" s="11"/>
     </x:row>
     <x:row r="218">
       <x:c r="A218" s="9"/>
@@ -2388,7 +2168,6 @@
       <x:c r="E218" s="9"/>
       <x:c r="G218" s="9"/>
       <x:c r="H218" s="9"/>
-      <x:c r="K218" s="11"/>
     </x:row>
     <x:row r="219">
       <x:c r="A219" s="9"/>
@@ -2397,7 +2176,6 @@
       <x:c r="E219" s="9"/>
       <x:c r="G219" s="9"/>
       <x:c r="H219" s="9"/>
-      <x:c r="K219" s="11"/>
     </x:row>
     <x:row r="220">
       <x:c r="A220" s="9"/>
@@ -2406,7 +2184,6 @@
       <x:c r="E220" s="9"/>
       <x:c r="G220" s="9"/>
       <x:c r="H220" s="9"/>
-      <x:c r="K220" s="11"/>
     </x:row>
     <x:row r="221">
       <x:c r="A221" s="9"/>
@@ -2415,7 +2192,6 @@
       <x:c r="E221" s="9"/>
       <x:c r="G221" s="9"/>
       <x:c r="H221" s="9"/>
-      <x:c r="K221" s="11"/>
     </x:row>
     <x:row r="222">
       <x:c r="A222" s="9"/>
@@ -2424,7 +2200,6 @@
       <x:c r="E222" s="9"/>
       <x:c r="G222" s="9"/>
       <x:c r="H222" s="9"/>
-      <x:c r="K222" s="11"/>
     </x:row>
     <x:row r="223">
       <x:c r="A223" s="9"/>
@@ -2433,7 +2208,6 @@
       <x:c r="E223" s="9"/>
       <x:c r="G223" s="9"/>
       <x:c r="H223" s="9"/>
-      <x:c r="K223" s="11"/>
     </x:row>
     <x:row r="224">
       <x:c r="A224" s="9"/>
@@ -2442,7 +2216,6 @@
       <x:c r="E224" s="9"/>
       <x:c r="G224" s="9"/>
       <x:c r="H224" s="9"/>
-      <x:c r="K224" s="11"/>
     </x:row>
     <x:row r="225">
       <x:c r="A225" s="9"/>
@@ -2451,7 +2224,6 @@
       <x:c r="E225" s="9"/>
       <x:c r="G225" s="9"/>
       <x:c r="H225" s="9"/>
-      <x:c r="K225" s="11"/>
     </x:row>
     <x:row r="226">
       <x:c r="A226" s="9"/>
@@ -2460,7 +2232,6 @@
       <x:c r="E226" s="9"/>
       <x:c r="G226" s="9"/>
       <x:c r="H226" s="9"/>
-      <x:c r="K226" s="11"/>
     </x:row>
     <x:row r="227">
       <x:c r="A227" s="9"/>
@@ -2469,7 +2240,6 @@
       <x:c r="E227" s="9"/>
       <x:c r="G227" s="9"/>
       <x:c r="H227" s="9"/>
-      <x:c r="K227" s="11"/>
     </x:row>
     <x:row r="228">
       <x:c r="A228" s="9"/>
@@ -2478,7 +2248,6 @@
       <x:c r="E228" s="9"/>
       <x:c r="G228" s="9"/>
       <x:c r="H228" s="9"/>
-      <x:c r="K228" s="11"/>
     </x:row>
     <x:row r="229">
       <x:c r="A229" s="9"/>
@@ -2487,7 +2256,6 @@
       <x:c r="E229" s="9"/>
       <x:c r="G229" s="9"/>
       <x:c r="H229" s="9"/>
-      <x:c r="K229" s="11"/>
     </x:row>
     <x:row r="230">
       <x:c r="A230" s="9"/>
@@ -2496,7 +2264,6 @@
       <x:c r="E230" s="9"/>
       <x:c r="G230" s="9"/>
       <x:c r="H230" s="9"/>
-      <x:c r="K230" s="11"/>
     </x:row>
     <x:row r="231">
       <x:c r="A231" s="9"/>
@@ -2505,7 +2272,6 @@
       <x:c r="E231" s="9"/>
       <x:c r="G231" s="9"/>
       <x:c r="H231" s="9"/>
-      <x:c r="K231" s="11"/>
     </x:row>
     <x:row r="232">
       <x:c r="A232" s="9"/>
@@ -2514,7 +2280,6 @@
       <x:c r="E232" s="9"/>
       <x:c r="G232" s="9"/>
       <x:c r="H232" s="9"/>
-      <x:c r="K232" s="11"/>
     </x:row>
     <x:row r="233">
       <x:c r="A233" s="9"/>
@@ -2523,7 +2288,6 @@
       <x:c r="E233" s="9"/>
       <x:c r="G233" s="9"/>
       <x:c r="H233" s="9"/>
-      <x:c r="K233" s="11"/>
     </x:row>
     <x:row r="234">
       <x:c r="A234" s="9"/>
@@ -2532,7 +2296,6 @@
       <x:c r="E234" s="9"/>
       <x:c r="G234" s="9"/>
       <x:c r="H234" s="9"/>
-      <x:c r="K234" s="11"/>
     </x:row>
     <x:row r="235">
       <x:c r="A235" s="9"/>
@@ -2541,7 +2304,6 @@
       <x:c r="E235" s="9"/>
       <x:c r="G235" s="9"/>
       <x:c r="H235" s="9"/>
-      <x:c r="K235" s="11"/>
     </x:row>
     <x:row r="236">
       <x:c r="A236" s="9"/>
@@ -2550,7 +2312,6 @@
       <x:c r="E236" s="9"/>
       <x:c r="G236" s="9"/>
       <x:c r="H236" s="9"/>
-      <x:c r="K236" s="11"/>
     </x:row>
     <x:row r="237">
       <x:c r="A237" s="9"/>
@@ -2559,7 +2320,6 @@
       <x:c r="E237" s="9"/>
       <x:c r="G237" s="9"/>
       <x:c r="H237" s="9"/>
-      <x:c r="K237" s="11"/>
     </x:row>
     <x:row r="238">
       <x:c r="A238" s="9"/>
@@ -2568,7 +2328,6 @@
       <x:c r="E238" s="9"/>
       <x:c r="G238" s="9"/>
       <x:c r="H238" s="9"/>
-      <x:c r="K238" s="11"/>
     </x:row>
     <x:row r="239">
       <x:c r="A239" s="9"/>
@@ -2577,7 +2336,6 @@
       <x:c r="E239" s="9"/>
       <x:c r="G239" s="9"/>
       <x:c r="H239" s="9"/>
-      <x:c r="K239" s="11"/>
     </x:row>
     <x:row r="240">
       <x:c r="A240" s="9"/>
@@ -2586,7 +2344,6 @@
       <x:c r="E240" s="9"/>
       <x:c r="G240" s="9"/>
       <x:c r="H240" s="9"/>
-      <x:c r="K240" s="11"/>
     </x:row>
     <x:row r="241">
       <x:c r="A241" s="9"/>
@@ -2595,7 +2352,6 @@
       <x:c r="E241" s="9"/>
       <x:c r="G241" s="9"/>
       <x:c r="H241" s="9"/>
-      <x:c r="K241" s="11"/>
     </x:row>
     <x:row r="242">
       <x:c r="A242" s="9"/>
@@ -2604,7 +2360,6 @@
       <x:c r="E242" s="9"/>
       <x:c r="G242" s="9"/>
       <x:c r="H242" s="9"/>
-      <x:c r="K242" s="11"/>
     </x:row>
     <x:row r="243">
       <x:c r="A243" s="9"/>
@@ -2613,7 +2368,6 @@
       <x:c r="E243" s="9"/>
       <x:c r="G243" s="9"/>
       <x:c r="H243" s="9"/>
-      <x:c r="K243" s="11"/>
     </x:row>
     <x:row r="244">
       <x:c r="A244" s="9"/>
@@ -2622,7 +2376,6 @@
       <x:c r="E244" s="9"/>
       <x:c r="G244" s="9"/>
       <x:c r="H244" s="9"/>
-      <x:c r="K244" s="11"/>
     </x:row>
     <x:row r="245">
       <x:c r="A245" s="9"/>
@@ -2631,7 +2384,6 @@
       <x:c r="E245" s="9"/>
       <x:c r="G245" s="9"/>
       <x:c r="H245" s="9"/>
-      <x:c r="K245" s="11"/>
     </x:row>
     <x:row r="246">
       <x:c r="A246" s="9"/>
@@ -2640,7 +2392,6 @@
       <x:c r="E246" s="9"/>
       <x:c r="G246" s="9"/>
       <x:c r="H246" s="9"/>
-      <x:c r="K246" s="11"/>
     </x:row>
     <x:row r="247">
       <x:c r="A247" s="9"/>
@@ -2649,7 +2400,6 @@
       <x:c r="E247" s="9"/>
       <x:c r="G247" s="9"/>
       <x:c r="H247" s="9"/>
-      <x:c r="K247" s="11"/>
     </x:row>
     <x:row r="248">
       <x:c r="A248" s="9"/>
@@ -2658,7 +2408,6 @@
       <x:c r="E248" s="9"/>
       <x:c r="G248" s="9"/>
       <x:c r="H248" s="9"/>
-      <x:c r="K248" s="11"/>
     </x:row>
     <x:row r="249">
       <x:c r="A249" s="9"/>
@@ -2667,7 +2416,6 @@
       <x:c r="E249" s="9"/>
       <x:c r="G249" s="9"/>
       <x:c r="H249" s="9"/>
-      <x:c r="K249" s="11"/>
     </x:row>
     <x:row r="250">
       <x:c r="A250" s="9"/>
@@ -2676,7 +2424,6 @@
       <x:c r="E250" s="9"/>
       <x:c r="G250" s="9"/>
       <x:c r="H250" s="9"/>
-      <x:c r="K250" s="11"/>
     </x:row>
     <x:row r="251">
       <x:c r="A251" s="9"/>
@@ -2685,7 +2432,6 @@
       <x:c r="E251" s="9"/>
       <x:c r="G251" s="9"/>
       <x:c r="H251" s="9"/>
-      <x:c r="K251" s="11"/>
     </x:row>
     <x:row r="252">
       <x:c r="A252" s="9"/>
@@ -2694,7 +2440,6 @@
       <x:c r="E252" s="9"/>
       <x:c r="G252" s="9"/>
       <x:c r="H252" s="9"/>
-      <x:c r="K252" s="11"/>
     </x:row>
     <x:row r="253">
       <x:c r="A253" s="9"/>
@@ -2703,7 +2448,6 @@
       <x:c r="E253" s="9"/>
       <x:c r="G253" s="9"/>
       <x:c r="H253" s="9"/>
-      <x:c r="K253" s="11"/>
     </x:row>
     <x:row r="254">
       <x:c r="A254" s="9"/>
@@ -2712,7 +2456,6 @@
       <x:c r="E254" s="9"/>
       <x:c r="G254" s="9"/>
       <x:c r="H254" s="9"/>
-      <x:c r="K254" s="11"/>
     </x:row>
     <x:row r="255">
       <x:c r="A255" s="9"/>
@@ -2721,7 +2464,6 @@
       <x:c r="E255" s="9"/>
       <x:c r="G255" s="9"/>
       <x:c r="H255" s="9"/>
-      <x:c r="K255" s="11"/>
     </x:row>
     <x:row r="256">
       <x:c r="A256" s="9"/>
@@ -2730,7 +2472,6 @@
       <x:c r="E256" s="9"/>
       <x:c r="G256" s="9"/>
       <x:c r="H256" s="9"/>
-      <x:c r="K256" s="11"/>
     </x:row>
     <x:row r="257">
       <x:c r="A257" s="9"/>
@@ -2739,7 +2480,6 @@
       <x:c r="E257" s="9"/>
       <x:c r="G257" s="9"/>
       <x:c r="H257" s="9"/>
-      <x:c r="K257" s="11"/>
     </x:row>
     <x:row r="258">
       <x:c r="A258" s="9"/>
@@ -2748,7 +2488,6 @@
       <x:c r="E258" s="9"/>
       <x:c r="G258" s="9"/>
       <x:c r="H258" s="9"/>
-      <x:c r="K258" s="11"/>
     </x:row>
     <x:row r="259">
       <x:c r="A259" s="9"/>
@@ -2757,7 +2496,6 @@
       <x:c r="E259" s="9"/>
       <x:c r="G259" s="9"/>
       <x:c r="H259" s="9"/>
-      <x:c r="K259" s="11"/>
     </x:row>
     <x:row r="260">
       <x:c r="A260" s="9"/>
@@ -2766,7 +2504,6 @@
       <x:c r="E260" s="9"/>
       <x:c r="G260" s="9"/>
       <x:c r="H260" s="9"/>
-      <x:c r="K260" s="11"/>
     </x:row>
     <x:row r="261">
       <x:c r="A261" s="9"/>
@@ -2775,7 +2512,6 @@
       <x:c r="E261" s="9"/>
       <x:c r="G261" s="9"/>
       <x:c r="H261" s="9"/>
-      <x:c r="K261" s="11"/>
     </x:row>
     <x:row r="262">
       <x:c r="A262" s="9"/>
@@ -2784,7 +2520,6 @@
       <x:c r="E262" s="9"/>
       <x:c r="G262" s="9"/>
       <x:c r="H262" s="9"/>
-      <x:c r="K262" s="11"/>
     </x:row>
     <x:row r="263">
       <x:c r="A263" s="9"/>
@@ -2793,7 +2528,6 @@
       <x:c r="E263" s="9"/>
       <x:c r="G263" s="9"/>
       <x:c r="H263" s="9"/>
-      <x:c r="K263" s="11"/>
     </x:row>
     <x:row r="264">
       <x:c r="A264" s="9"/>
@@ -2802,7 +2536,6 @@
       <x:c r="E264" s="9"/>
       <x:c r="G264" s="9"/>
       <x:c r="H264" s="9"/>
-      <x:c r="K264" s="11"/>
     </x:row>
     <x:row r="265">
       <x:c r="A265" s="9"/>
@@ -2811,7 +2544,6 @@
       <x:c r="E265" s="9"/>
       <x:c r="G265" s="9"/>
       <x:c r="H265" s="9"/>
-      <x:c r="K265" s="11"/>
     </x:row>
     <x:row r="266">
       <x:c r="A266" s="9"/>
@@ -2820,7 +2552,6 @@
       <x:c r="E266" s="9"/>
       <x:c r="G266" s="9"/>
       <x:c r="H266" s="9"/>
-      <x:c r="K266" s="11"/>
     </x:row>
     <x:row r="267">
       <x:c r="A267" s="9"/>
@@ -2829,7 +2560,6 @@
       <x:c r="E267" s="9"/>
       <x:c r="G267" s="9"/>
       <x:c r="H267" s="9"/>
-      <x:c r="K267" s="11"/>
     </x:row>
     <x:row r="268">
       <x:c r="A268" s="9"/>
@@ -2838,7 +2568,6 @@
       <x:c r="E268" s="9"/>
       <x:c r="G268" s="9"/>
       <x:c r="H268" s="9"/>
-      <x:c r="K268" s="11"/>
     </x:row>
     <x:row r="269">
       <x:c r="A269" s="9"/>
@@ -2847,7 +2576,6 @@
       <x:c r="E269" s="9"/>
       <x:c r="G269" s="9"/>
       <x:c r="H269" s="9"/>
-      <x:c r="K269" s="11"/>
     </x:row>
     <x:row r="270">
       <x:c r="A270" s="9"/>
@@ -2856,7 +2584,6 @@
       <x:c r="E270" s="9"/>
       <x:c r="G270" s="9"/>
       <x:c r="H270" s="9"/>
-      <x:c r="K270" s="11"/>
     </x:row>
     <x:row r="271">
       <x:c r="A271" s="9"/>
@@ -2865,7 +2592,6 @@
       <x:c r="E271" s="9"/>
       <x:c r="G271" s="9"/>
       <x:c r="H271" s="9"/>
-      <x:c r="K271" s="11"/>
     </x:row>
     <x:row r="272">
       <x:c r="A272" s="9"/>
@@ -2874,7 +2600,6 @@
       <x:c r="E272" s="9"/>
       <x:c r="G272" s="9"/>
       <x:c r="H272" s="9"/>
-      <x:c r="K272" s="11"/>
     </x:row>
     <x:row r="273">
       <x:c r="A273" s="9"/>
@@ -2883,7 +2608,6 @@
       <x:c r="E273" s="9"/>
       <x:c r="G273" s="9"/>
       <x:c r="H273" s="9"/>
-      <x:c r="K273" s="11"/>
     </x:row>
     <x:row r="274">
       <x:c r="A274" s="9"/>
@@ -2892,7 +2616,6 @@
       <x:c r="E274" s="9"/>
       <x:c r="G274" s="9"/>
       <x:c r="H274" s="9"/>
-      <x:c r="K274" s="11"/>
     </x:row>
     <x:row r="275">
       <x:c r="A275" s="9"/>
@@ -2901,7 +2624,6 @@
       <x:c r="E275" s="9"/>
       <x:c r="G275" s="9"/>
       <x:c r="H275" s="9"/>
-      <x:c r="K275" s="11"/>
     </x:row>
     <x:row r="276">
       <x:c r="A276" s="9"/>
@@ -2910,7 +2632,6 @@
       <x:c r="E276" s="9"/>
       <x:c r="G276" s="9"/>
       <x:c r="H276" s="9"/>
-      <x:c r="K276" s="11"/>
     </x:row>
     <x:row r="277">
       <x:c r="A277" s="9"/>
@@ -2919,7 +2640,6 @@
       <x:c r="E277" s="9"/>
       <x:c r="G277" s="9"/>
       <x:c r="H277" s="9"/>
-      <x:c r="K277" s="11"/>
     </x:row>
     <x:row r="278">
       <x:c r="A278" s="9"/>
@@ -2928,7 +2648,6 @@
       <x:c r="E278" s="9"/>
       <x:c r="G278" s="9"/>
       <x:c r="H278" s="9"/>
-      <x:c r="K278" s="11"/>
     </x:row>
     <x:row r="279">
       <x:c r="A279" s="9"/>
@@ -2937,7 +2656,6 @@
       <x:c r="E279" s="9"/>
       <x:c r="G279" s="9"/>
       <x:c r="H279" s="9"/>
-      <x:c r="K279" s="11"/>
     </x:row>
     <x:row r="280">
       <x:c r="A280" s="9"/>
@@ -2946,7 +2664,6 @@
       <x:c r="E280" s="9"/>
       <x:c r="G280" s="9"/>
       <x:c r="H280" s="9"/>
-      <x:c r="K280" s="11"/>
     </x:row>
     <x:row r="281">
       <x:c r="A281" s="9"/>
@@ -2955,7 +2672,6 @@
       <x:c r="E281" s="9"/>
       <x:c r="G281" s="9"/>
       <x:c r="H281" s="9"/>
-      <x:c r="K281" s="11"/>
     </x:row>
     <x:row r="282">
       <x:c r="A282" s="9"/>
@@ -2964,7 +2680,6 @@
       <x:c r="E282" s="9"/>
       <x:c r="G282" s="9"/>
       <x:c r="H282" s="9"/>
-      <x:c r="K282" s="11"/>
     </x:row>
     <x:row r="283">
       <x:c r="A283" s="9"/>
@@ -2973,7 +2688,6 @@
       <x:c r="E283" s="9"/>
       <x:c r="G283" s="9"/>
       <x:c r="H283" s="9"/>
-      <x:c r="K283" s="11"/>
     </x:row>
     <x:row r="284">
       <x:c r="A284" s="9"/>
@@ -2982,7 +2696,6 @@
       <x:c r="E284" s="9"/>
       <x:c r="G284" s="9"/>
       <x:c r="H284" s="9"/>
-      <x:c r="K284" s="11"/>
     </x:row>
     <x:row r="285">
       <x:c r="A285" s="9"/>
@@ -2991,7 +2704,6 @@
       <x:c r="E285" s="9"/>
       <x:c r="G285" s="9"/>
       <x:c r="H285" s="9"/>
-      <x:c r="K285" s="11"/>
     </x:row>
     <x:row r="286">
       <x:c r="A286" s="9"/>
@@ -3000,7 +2712,6 @@
       <x:c r="E286" s="9"/>
       <x:c r="G286" s="9"/>
       <x:c r="H286" s="9"/>
-      <x:c r="K286" s="11"/>
     </x:row>
     <x:row r="287">
       <x:c r="A287" s="9"/>
@@ -3009,7 +2720,6 @@
       <x:c r="E287" s="9"/>
       <x:c r="G287" s="9"/>
       <x:c r="H287" s="9"/>
-      <x:c r="K287" s="11"/>
     </x:row>
     <x:row r="288">
       <x:c r="A288" s="9"/>
@@ -3018,7 +2728,6 @@
       <x:c r="E288" s="9"/>
       <x:c r="G288" s="9"/>
       <x:c r="H288" s="9"/>
-      <x:c r="K288" s="11"/>
     </x:row>
     <x:row r="289">
       <x:c r="A289" s="9"/>
@@ -3027,7 +2736,6 @@
       <x:c r="E289" s="9"/>
       <x:c r="G289" s="9"/>
       <x:c r="H289" s="9"/>
-      <x:c r="K289" s="11"/>
     </x:row>
     <x:row r="290">
       <x:c r="A290" s="9"/>
@@ -3036,7 +2744,6 @@
       <x:c r="E290" s="9"/>
       <x:c r="G290" s="9"/>
       <x:c r="H290" s="9"/>
-      <x:c r="K290" s="11"/>
     </x:row>
     <x:row r="291">
       <x:c r="A291" s="9"/>
@@ -3045,7 +2752,6 @@
       <x:c r="E291" s="9"/>
       <x:c r="G291" s="9"/>
       <x:c r="H291" s="9"/>
-      <x:c r="K291" s="11"/>
     </x:row>
     <x:row r="292">
       <x:c r="A292" s="9"/>
@@ -3054,7 +2760,6 @@
       <x:c r="E292" s="9"/>
       <x:c r="G292" s="9"/>
       <x:c r="H292" s="9"/>
-      <x:c r="K292" s="11"/>
     </x:row>
     <x:row r="293">
       <x:c r="A293" s="9"/>
@@ -3063,7 +2768,6 @@
       <x:c r="E293" s="9"/>
       <x:c r="G293" s="9"/>
       <x:c r="H293" s="9"/>
-      <x:c r="K293" s="11"/>
     </x:row>
     <x:row r="294">
       <x:c r="A294" s="9"/>
@@ -3072,7 +2776,6 @@
       <x:c r="E294" s="9"/>
       <x:c r="G294" s="9"/>
       <x:c r="H294" s="9"/>
-      <x:c r="K294" s="11"/>
     </x:row>
     <x:row r="295">
       <x:c r="A295" s="9"/>
@@ -3081,7 +2784,6 @@
       <x:c r="E295" s="9"/>
       <x:c r="G295" s="9"/>
       <x:c r="H295" s="9"/>
-      <x:c r="K295" s="11"/>
     </x:row>
     <x:row r="296">
       <x:c r="A296" s="9"/>
@@ -3090,7 +2792,6 @@
       <x:c r="E296" s="9"/>
       <x:c r="G296" s="9"/>
       <x:c r="H296" s="9"/>
-      <x:c r="K296" s="11"/>
     </x:row>
     <x:row r="297">
       <x:c r="A297" s="9"/>
@@ -3099,7 +2800,6 @@
       <x:c r="E297" s="9"/>
       <x:c r="G297" s="9"/>
       <x:c r="H297" s="9"/>
-      <x:c r="K297" s="11"/>
     </x:row>
     <x:row r="298">
       <x:c r="A298" s="9"/>
@@ -3108,7 +2808,6 @@
       <x:c r="E298" s="9"/>
       <x:c r="G298" s="9"/>
       <x:c r="H298" s="9"/>
-      <x:c r="K298" s="11"/>
     </x:row>
     <x:row r="299">
       <x:c r="A299" s="9"/>
@@ -3117,7 +2816,6 @@
       <x:c r="E299" s="9"/>
       <x:c r="G299" s="9"/>
       <x:c r="H299" s="9"/>
-      <x:c r="K299" s="11"/>
     </x:row>
     <x:row r="300">
       <x:c r="A300" s="9"/>
@@ -3126,7 +2824,6 @@
       <x:c r="E300" s="9"/>
       <x:c r="G300" s="9"/>
       <x:c r="H300" s="9"/>
-      <x:c r="K300" s="11"/>
     </x:row>
     <x:row r="301">
       <x:c r="A301" s="9"/>
@@ -3135,7 +2832,6 @@
       <x:c r="E301" s="9"/>
       <x:c r="G301" s="9"/>
       <x:c r="H301" s="9"/>
-      <x:c r="K301" s="11"/>
     </x:row>
     <x:row r="302">
       <x:c r="A302" s="9"/>
@@ -3144,7 +2840,6 @@
       <x:c r="E302" s="9"/>
       <x:c r="G302" s="9"/>
       <x:c r="H302" s="9"/>
-      <x:c r="K302" s="11"/>
     </x:row>
     <x:row r="303">
       <x:c r="A303" s="9"/>
@@ -3153,7 +2848,6 @@
       <x:c r="E303" s="9"/>
       <x:c r="G303" s="9"/>
       <x:c r="H303" s="9"/>
-      <x:c r="K303" s="11"/>
     </x:row>
     <x:row r="304">
       <x:c r="A304" s="9"/>
@@ -3162,7 +2856,6 @@
       <x:c r="E304" s="9"/>
       <x:c r="G304" s="9"/>
       <x:c r="H304" s="9"/>
-      <x:c r="K304" s="11"/>
     </x:row>
     <x:row r="305">
       <x:c r="A305" s="9"/>
@@ -3171,7 +2864,6 @@
       <x:c r="E305" s="9"/>
       <x:c r="G305" s="9"/>
       <x:c r="H305" s="9"/>
-      <x:c r="K305" s="11"/>
     </x:row>
     <x:row r="306">
       <x:c r="A306" s="9"/>
@@ -3180,7 +2872,6 @@
       <x:c r="E306" s="9"/>
       <x:c r="G306" s="9"/>
       <x:c r="H306" s="9"/>
-      <x:c r="K306" s="11"/>
     </x:row>
     <x:row r="307">
       <x:c r="A307" s="9"/>
@@ -3189,7 +2880,6 @@
       <x:c r="E307" s="9"/>
       <x:c r="G307" s="9"/>
       <x:c r="H307" s="9"/>
-      <x:c r="K307" s="11"/>
     </x:row>
     <x:row r="308">
       <x:c r="A308" s="9"/>
@@ -3198,7 +2888,6 @@
       <x:c r="E308" s="9"/>
       <x:c r="G308" s="9"/>
       <x:c r="H308" s="9"/>
-      <x:c r="K308" s="11"/>
     </x:row>
     <x:row r="309">
       <x:c r="A309" s="9"/>
@@ -3207,7 +2896,6 @@
       <x:c r="E309" s="9"/>
       <x:c r="G309" s="9"/>
       <x:c r="H309" s="9"/>
-      <x:c r="K309" s="11"/>
     </x:row>
     <x:row r="310">
       <x:c r="A310" s="9"/>
@@ -3216,7 +2904,6 @@
       <x:c r="E310" s="9"/>
       <x:c r="G310" s="9"/>
       <x:c r="H310" s="9"/>
-      <x:c r="K310" s="11"/>
     </x:row>
     <x:row r="311">
       <x:c r="A311" s="9"/>
@@ -3225,7 +2912,6 @@
       <x:c r="E311" s="9"/>
       <x:c r="G311" s="9"/>
       <x:c r="H311" s="9"/>
-      <x:c r="K311" s="11"/>
     </x:row>
     <x:row r="312">
       <x:c r="A312" s="9"/>
@@ -3234,7 +2920,6 @@
       <x:c r="E312" s="9"/>
       <x:c r="G312" s="9"/>
       <x:c r="H312" s="9"/>
-      <x:c r="K312" s="11"/>
     </x:row>
     <x:row r="313">
       <x:c r="A313" s="9"/>
@@ -3243,7 +2928,6 @@
       <x:c r="E313" s="9"/>
       <x:c r="G313" s="9"/>
       <x:c r="H313" s="9"/>
-      <x:c r="K313" s="11"/>
     </x:row>
     <x:row r="314">
       <x:c r="A314" s="9"/>
@@ -3252,7 +2936,6 @@
       <x:c r="E314" s="9"/>
       <x:c r="G314" s="9"/>
       <x:c r="H314" s="9"/>
-      <x:c r="K314" s="11"/>
     </x:row>
     <x:row r="315">
       <x:c r="A315" s="9"/>
@@ -3261,7 +2944,6 @@
       <x:c r="E315" s="9"/>
       <x:c r="G315" s="9"/>
       <x:c r="H315" s="9"/>
-      <x:c r="K315" s="11"/>
     </x:row>
     <x:row r="316">
       <x:c r="A316" s="9"/>
@@ -3270,7 +2952,6 @@
       <x:c r="E316" s="9"/>
       <x:c r="G316" s="9"/>
       <x:c r="H316" s="9"/>
-      <x:c r="K316" s="11"/>
     </x:row>
     <x:row r="317">
       <x:c r="A317" s="9"/>
@@ -3279,7 +2960,6 @@
       <x:c r="E317" s="9"/>
       <x:c r="G317" s="9"/>
       <x:c r="H317" s="9"/>
-      <x:c r="K317" s="11"/>
     </x:row>
     <x:row r="318">
       <x:c r="A318" s="9"/>
@@ -3288,7 +2968,6 @@
       <x:c r="E318" s="9"/>
       <x:c r="G318" s="9"/>
       <x:c r="H318" s="9"/>
-      <x:c r="K318" s="11"/>
     </x:row>
     <x:row r="319">
       <x:c r="A319" s="9"/>
@@ -3297,7 +2976,6 @@
       <x:c r="E319" s="9"/>
       <x:c r="G319" s="9"/>
       <x:c r="H319" s="9"/>
-      <x:c r="K319" s="11"/>
     </x:row>
     <x:row r="320">
       <x:c r="A320" s="9"/>
@@ -3306,7 +2984,6 @@
       <x:c r="E320" s="9"/>
       <x:c r="G320" s="9"/>
       <x:c r="H320" s="9"/>
-      <x:c r="K320" s="11"/>
     </x:row>
     <x:row r="321">
       <x:c r="A321" s="9"/>
@@ -3315,7 +2992,6 @@
       <x:c r="E321" s="9"/>
       <x:c r="G321" s="9"/>
       <x:c r="H321" s="9"/>
-      <x:c r="K321" s="11"/>
     </x:row>
     <x:row r="322">
       <x:c r="A322" s="9"/>
@@ -3324,7 +3000,6 @@
       <x:c r="E322" s="9"/>
       <x:c r="G322" s="9"/>
       <x:c r="H322" s="9"/>
-      <x:c r="K322" s="11"/>
     </x:row>
     <x:row r="323">
       <x:c r="A323" s="9"/>
@@ -3333,7 +3008,6 @@
       <x:c r="E323" s="9"/>
       <x:c r="G323" s="9"/>
       <x:c r="H323" s="9"/>
-      <x:c r="K323" s="11"/>
     </x:row>
     <x:row r="324">
       <x:c r="A324" s="9"/>
@@ -3342,7 +3016,6 @@
       <x:c r="E324" s="9"/>
       <x:c r="G324" s="9"/>
       <x:c r="H324" s="9"/>
-      <x:c r="K324" s="11"/>
     </x:row>
     <x:row r="325">
       <x:c r="A325" s="9"/>
@@ -3351,7 +3024,6 @@
       <x:c r="E325" s="9"/>
       <x:c r="G325" s="9"/>
       <x:c r="H325" s="9"/>
-      <x:c r="K325" s="11"/>
     </x:row>
     <x:row r="326">
       <x:c r="A326" s="9"/>
@@ -3360,7 +3032,6 @@
       <x:c r="E326" s="9"/>
       <x:c r="G326" s="9"/>
       <x:c r="H326" s="9"/>
-      <x:c r="K326" s="11"/>
     </x:row>
     <x:row r="327">
       <x:c r="A327" s="9"/>
@@ -3369,7 +3040,6 @@
       <x:c r="E327" s="9"/>
       <x:c r="G327" s="9"/>
       <x:c r="H327" s="9"/>
-      <x:c r="K327" s="11"/>
     </x:row>
     <x:row r="328">
       <x:c r="A328" s="9"/>
@@ -3378,7 +3048,6 @@
       <x:c r="E328" s="9"/>
       <x:c r="G328" s="9"/>
       <x:c r="H328" s="9"/>
-      <x:c r="K328" s="11"/>
     </x:row>
     <x:row r="329">
       <x:c r="A329" s="9"/>
@@ -3387,7 +3056,6 @@
       <x:c r="E329" s="9"/>
       <x:c r="G329" s="9"/>
       <x:c r="H329" s="9"/>
-      <x:c r="K329" s="11"/>
     </x:row>
     <x:row r="330">
       <x:c r="A330" s="9"/>
@@ -3396,7 +3064,6 @@
       <x:c r="E330" s="9"/>
       <x:c r="G330" s="9"/>
       <x:c r="H330" s="9"/>
-      <x:c r="K330" s="11"/>
     </x:row>
     <x:row r="331">
       <x:c r="A331" s="9"/>
@@ -3405,7 +3072,6 @@
       <x:c r="E331" s="9"/>
       <x:c r="G331" s="9"/>
       <x:c r="H331" s="9"/>
-      <x:c r="K331" s="11"/>
     </x:row>
     <x:row r="332">
       <x:c r="A332" s="9"/>
@@ -3414,7 +3080,6 @@
       <x:c r="E332" s="9"/>
       <x:c r="G332" s="9"/>
       <x:c r="H332" s="9"/>
-      <x:c r="K332" s="11"/>
     </x:row>
     <x:row r="333">
       <x:c r="A333" s="9"/>
@@ -3423,7 +3088,6 @@
       <x:c r="E333" s="9"/>
       <x:c r="G333" s="9"/>
       <x:c r="H333" s="9"/>
-      <x:c r="K333" s="11"/>
     </x:row>
     <x:row r="334">
       <x:c r="A334" s="9"/>
@@ -3432,7 +3096,6 @@
       <x:c r="E334" s="9"/>
       <x:c r="G334" s="9"/>
       <x:c r="H334" s="9"/>
-      <x:c r="K334" s="11"/>
     </x:row>
     <x:row r="335">
       <x:c r="A335" s="9"/>
@@ -3441,7 +3104,6 @@
       <x:c r="E335" s="9"/>
       <x:c r="G335" s="9"/>
       <x:c r="H335" s="9"/>
-      <x:c r="K335" s="11"/>
     </x:row>
     <x:row r="336">
       <x:c r="A336" s="9"/>
@@ -3450,7 +3112,6 @@
       <x:c r="E336" s="9"/>
       <x:c r="G336" s="9"/>
       <x:c r="H336" s="9"/>
-      <x:c r="K336" s="11"/>
     </x:row>
     <x:row r="337">
       <x:c r="A337" s="9"/>
@@ -3459,7 +3120,6 @@
       <x:c r="E337" s="9"/>
       <x:c r="G337" s="9"/>
       <x:c r="H337" s="9"/>
-      <x:c r="K337" s="11"/>
     </x:row>
     <x:row r="338">
       <x:c r="A338" s="9"/>
@@ -3468,7 +3128,6 @@
       <x:c r="E338" s="9"/>
       <x:c r="G338" s="9"/>
       <x:c r="H338" s="9"/>
-      <x:c r="K338" s="11"/>
     </x:row>
     <x:row r="339">
       <x:c r="A339" s="9"/>
@@ -3477,7 +3136,6 @@
       <x:c r="E339" s="9"/>
       <x:c r="G339" s="9"/>
       <x:c r="H339" s="9"/>
-      <x:c r="K339" s="11"/>
     </x:row>
     <x:row r="340">
       <x:c r="A340" s="9"/>
@@ -3486,7 +3144,6 @@
       <x:c r="E340" s="9"/>
       <x:c r="G340" s="9"/>
       <x:c r="H340" s="9"/>
-      <x:c r="K340" s="11"/>
     </x:row>
     <x:row r="341">
       <x:c r="A341" s="9"/>
@@ -3495,7 +3152,6 @@
       <x:c r="E341" s="9"/>
       <x:c r="G341" s="9"/>
       <x:c r="H341" s="9"/>
-      <x:c r="K341" s="11"/>
     </x:row>
     <x:row r="342">
       <x:c r="A342" s="9"/>
@@ -3504,7 +3160,6 @@
       <x:c r="E342" s="9"/>
       <x:c r="G342" s="9"/>
       <x:c r="H342" s="9"/>
-      <x:c r="K342" s="11"/>
     </x:row>
     <x:row r="343">
       <x:c r="A343" s="9"/>
@@ -3513,7 +3168,6 @@
       <x:c r="E343" s="9"/>
       <x:c r="G343" s="9"/>
       <x:c r="H343" s="9"/>
-      <x:c r="K343" s="11"/>
     </x:row>
     <x:row r="344">
       <x:c r="A344" s="9"/>
@@ -3522,7 +3176,6 @@
       <x:c r="E344" s="9"/>
       <x:c r="G344" s="9"/>
       <x:c r="H344" s="9"/>
-      <x:c r="K344" s="11"/>
     </x:row>
     <x:row r="345">
       <x:c r="A345" s="9"/>
@@ -3531,7 +3184,6 @@
       <x:c r="E345" s="9"/>
       <x:c r="G345" s="9"/>
       <x:c r="H345" s="9"/>
-      <x:c r="K345" s="11"/>
     </x:row>
     <x:row r="346">
       <x:c r="A346" s="9"/>
@@ -3540,7 +3192,6 @@
       <x:c r="E346" s="9"/>
       <x:c r="G346" s="9"/>
       <x:c r="H346" s="9"/>
-      <x:c r="K346" s="11"/>
     </x:row>
     <x:row r="347">
       <x:c r="A347" s="9"/>
@@ -3549,7 +3200,6 @@
       <x:c r="E347" s="9"/>
       <x:c r="G347" s="9"/>
       <x:c r="H347" s="9"/>
-      <x:c r="K347" s="11"/>
     </x:row>
     <x:row r="348">
       <x:c r="A348" s="9"/>
@@ -3558,7 +3208,6 @@
       <x:c r="E348" s="9"/>
       <x:c r="G348" s="9"/>
       <x:c r="H348" s="9"/>
-      <x:c r="K348" s="11"/>
     </x:row>
     <x:row r="349">
       <x:c r="A349" s="9"/>
@@ -3567,7 +3216,6 @@
       <x:c r="E349" s="9"/>
       <x:c r="G349" s="9"/>
       <x:c r="H349" s="9"/>
-      <x:c r="K349" s="11"/>
     </x:row>
     <x:row r="350">
       <x:c r="A350" s="9"/>
@@ -3576,7 +3224,6 @@
       <x:c r="E350" s="9"/>
       <x:c r="G350" s="9"/>
       <x:c r="H350" s="9"/>
-      <x:c r="K350" s="11"/>
     </x:row>
     <x:row r="351">
       <x:c r="A351" s="9"/>
@@ -3585,7 +3232,6 @@
       <x:c r="E351" s="9"/>
       <x:c r="G351" s="9"/>
       <x:c r="H351" s="9"/>
-      <x:c r="K351" s="11"/>
     </x:row>
     <x:row r="352">
       <x:c r="A352" s="9"/>
@@ -3594,7 +3240,6 @@
       <x:c r="E352" s="9"/>
       <x:c r="G352" s="9"/>
       <x:c r="H352" s="9"/>
-      <x:c r="K352" s="11"/>
     </x:row>
     <x:row r="353">
       <x:c r="A353" s="9"/>
@@ -3603,7 +3248,6 @@
       <x:c r="E353" s="9"/>
       <x:c r="G353" s="9"/>
       <x:c r="H353" s="9"/>
-      <x:c r="K353" s="11"/>
     </x:row>
     <x:row r="354">
       <x:c r="A354" s="9"/>
@@ -3612,7 +3256,6 @@
       <x:c r="E354" s="9"/>
       <x:c r="G354" s="9"/>
       <x:c r="H354" s="9"/>
-      <x:c r="K354" s="11"/>
     </x:row>
     <x:row r="355">
       <x:c r="A355" s="9"/>
@@ -3621,7 +3264,6 @@
       <x:c r="E355" s="9"/>
       <x:c r="G355" s="9"/>
       <x:c r="H355" s="9"/>
-      <x:c r="K355" s="11"/>
     </x:row>
     <x:row r="356">
       <x:c r="A356" s="9"/>
@@ -3630,7 +3272,6 @@
       <x:c r="E356" s="9"/>
       <x:c r="G356" s="9"/>
       <x:c r="H356" s="9"/>
-      <x:c r="K356" s="11"/>
     </x:row>
     <x:row r="357">
       <x:c r="A357" s="9"/>
@@ -3639,7 +3280,6 @@
       <x:c r="E357" s="9"/>
       <x:c r="G357" s="9"/>
       <x:c r="H357" s="9"/>
-      <x:c r="K357" s="11"/>
     </x:row>
     <x:row r="358">
       <x:c r="A358" s="9"/>
@@ -3648,7 +3288,6 @@
       <x:c r="E358" s="9"/>
       <x:c r="G358" s="9"/>
       <x:c r="H358" s="9"/>
-      <x:c r="K358" s="11"/>
     </x:row>
     <x:row r="359">
       <x:c r="A359" s="9"/>
@@ -3657,7 +3296,6 @@
       <x:c r="E359" s="9"/>
       <x:c r="G359" s="9"/>
       <x:c r="H359" s="9"/>
-      <x:c r="K359" s="11"/>
     </x:row>
     <x:row r="360">
       <x:c r="A360" s="9"/>
@@ -3666,7 +3304,6 @@
       <x:c r="E360" s="9"/>
       <x:c r="G360" s="9"/>
       <x:c r="H360" s="9"/>
-      <x:c r="K360" s="11"/>
     </x:row>
     <x:row r="361">
       <x:c r="A361" s="9"/>
@@ -3675,7 +3312,6 @@
       <x:c r="E361" s="9"/>
       <x:c r="G361" s="9"/>
       <x:c r="H361" s="9"/>
-      <x:c r="K361" s="11"/>
     </x:row>
     <x:row r="362">
       <x:c r="A362" s="9"/>
@@ -3684,7 +3320,6 @@
       <x:c r="E362" s="9"/>
       <x:c r="G362" s="9"/>
       <x:c r="H362" s="9"/>
-      <x:c r="K362" s="11"/>
     </x:row>
     <x:row r="363">
       <x:c r="A363" s="9"/>
@@ -3693,7 +3328,6 @@
       <x:c r="E363" s="9"/>
       <x:c r="G363" s="9"/>
       <x:c r="H363" s="9"/>
-      <x:c r="K363" s="11"/>
     </x:row>
     <x:row r="364">
       <x:c r="A364" s="9"/>
@@ -3702,7 +3336,6 @@
       <x:c r="E364" s="9"/>
       <x:c r="G364" s="9"/>
       <x:c r="H364" s="9"/>
-      <x:c r="K364" s="11"/>
     </x:row>
     <x:row r="365">
       <x:c r="A365" s="9"/>
@@ -3711,7 +3344,6 @@
       <x:c r="E365" s="9"/>
       <x:c r="G365" s="9"/>
       <x:c r="H365" s="9"/>
-      <x:c r="K365" s="11"/>
     </x:row>
     <x:row r="366">
       <x:c r="A366" s="9"/>
@@ -3720,7 +3352,6 @@
       <x:c r="E366" s="9"/>
       <x:c r="G366" s="9"/>
       <x:c r="H366" s="9"/>
-      <x:c r="K366" s="11"/>
     </x:row>
     <x:row r="367">
       <x:c r="A367" s="9"/>
@@ -3729,7 +3360,6 @@
       <x:c r="E367" s="9"/>
       <x:c r="G367" s="9"/>
       <x:c r="H367" s="9"/>
-      <x:c r="K367" s="11"/>
     </x:row>
     <x:row r="368">
       <x:c r="A368" s="9"/>
@@ -3738,7 +3368,6 @@
       <x:c r="E368" s="9"/>
       <x:c r="G368" s="9"/>
       <x:c r="H368" s="9"/>
-      <x:c r="K368" s="11"/>
     </x:row>
     <x:row r="369">
       <x:c r="A369" s="9"/>
@@ -3747,7 +3376,6 @@
       <x:c r="E369" s="9"/>
       <x:c r="G369" s="9"/>
       <x:c r="H369" s="9"/>
-      <x:c r="K369" s="11"/>
     </x:row>
     <x:row r="370">
       <x:c r="A370" s="9"/>
@@ -3756,7 +3384,6 @@
       <x:c r="E370" s="9"/>
       <x:c r="G370" s="9"/>
       <x:c r="H370" s="9"/>
-      <x:c r="K370" s="11"/>
     </x:row>
     <x:row r="371">
       <x:c r="A371" s="9"/>
@@ -3765,7 +3392,6 @@
       <x:c r="E371" s="9"/>
       <x:c r="G371" s="9"/>
       <x:c r="H371" s="9"/>
-      <x:c r="K371" s="11"/>
     </x:row>
     <x:row r="372">
       <x:c r="A372" s="9"/>
@@ -3774,7 +3400,6 @@
       <x:c r="E372" s="9"/>
       <x:c r="G372" s="9"/>
       <x:c r="H372" s="9"/>
-      <x:c r="K372" s="11"/>
     </x:row>
     <x:row r="373">
       <x:c r="A373" s="9"/>
@@ -3783,7 +3408,6 @@
       <x:c r="E373" s="9"/>
       <x:c r="G373" s="9"/>
       <x:c r="H373" s="9"/>
-      <x:c r="K373" s="11"/>
     </x:row>
     <x:row r="374">
       <x:c r="A374" s="9"/>
@@ -3792,7 +3416,6 @@
       <x:c r="E374" s="9"/>
       <x:c r="G374" s="9"/>
       <x:c r="H374" s="9"/>
-      <x:c r="K374" s="11"/>
     </x:row>
     <x:row r="375">
       <x:c r="A375" s="9"/>
@@ -3801,7 +3424,6 @@
       <x:c r="E375" s="9"/>
       <x:c r="G375" s="9"/>
       <x:c r="H375" s="9"/>
-      <x:c r="K375" s="11"/>
     </x:row>
     <x:row r="376">
       <x:c r="A376" s="9"/>
@@ -3810,7 +3432,6 @@
       <x:c r="E376" s="9"/>
       <x:c r="G376" s="9"/>
       <x:c r="H376" s="9"/>
-      <x:c r="K376" s="11"/>
     </x:row>
     <x:row r="377">
       <x:c r="A377" s="9"/>
@@ -3819,7 +3440,6 @@
       <x:c r="E377" s="9"/>
       <x:c r="G377" s="9"/>
       <x:c r="H377" s="9"/>
-      <x:c r="K377" s="11"/>
     </x:row>
     <x:row r="378">
       <x:c r="A378" s="9"/>
@@ -3828,7 +3448,6 @@
       <x:c r="E378" s="9"/>
       <x:c r="G378" s="9"/>
       <x:c r="H378" s="9"/>
-      <x:c r="K378" s="11"/>
     </x:row>
     <x:row r="379">
       <x:c r="A379" s="9"/>
@@ -3837,7 +3456,6 @@
       <x:c r="E379" s="9"/>
       <x:c r="G379" s="9"/>
       <x:c r="H379" s="9"/>
-      <x:c r="K379" s="11"/>
     </x:row>
     <x:row r="380">
       <x:c r="A380" s="9"/>
@@ -3846,7 +3464,6 @@
       <x:c r="E380" s="9"/>
       <x:c r="G380" s="9"/>
       <x:c r="H380" s="9"/>
-      <x:c r="K380" s="11"/>
     </x:row>
     <x:row r="381">
       <x:c r="A381" s="9"/>
@@ -3855,7 +3472,6 @@
       <x:c r="E381" s="9"/>
       <x:c r="G381" s="9"/>
       <x:c r="H381" s="9"/>
-      <x:c r="K381" s="11"/>
     </x:row>
     <x:row r="382">
       <x:c r="A382" s="9"/>
@@ -3864,7 +3480,6 @@
       <x:c r="E382" s="9"/>
       <x:c r="G382" s="9"/>
       <x:c r="H382" s="9"/>
-      <x:c r="K382" s="11"/>
     </x:row>
     <x:row r="383">
       <x:c r="A383" s="9"/>
@@ -3873,7 +3488,6 @@
       <x:c r="E383" s="9"/>
       <x:c r="G383" s="9"/>
       <x:c r="H383" s="9"/>
-      <x:c r="K383" s="11"/>
     </x:row>
     <x:row r="384">
       <x:c r="A384" s="9"/>
@@ -3882,7 +3496,6 @@
       <x:c r="E384" s="9"/>
       <x:c r="G384" s="9"/>
       <x:c r="H384" s="9"/>
-      <x:c r="K384" s="11"/>
     </x:row>
     <x:row r="385">
       <x:c r="A385" s="9"/>
@@ -3891,7 +3504,6 @@
       <x:c r="E385" s="9"/>
       <x:c r="G385" s="9"/>
       <x:c r="H385" s="9"/>
-      <x:c r="K385" s="11"/>
     </x:row>
     <x:row r="386">
       <x:c r="A386" s="9"/>
@@ -3900,7 +3512,6 @@
       <x:c r="E386" s="9"/>
       <x:c r="G386" s="9"/>
       <x:c r="H386" s="9"/>
-      <x:c r="K386" s="11"/>
     </x:row>
     <x:row r="387">
       <x:c r="A387" s="9"/>
@@ -3909,7 +3520,6 @@
       <x:c r="E387" s="9"/>
       <x:c r="G387" s="9"/>
       <x:c r="H387" s="9"/>
-      <x:c r="K387" s="11"/>
     </x:row>
     <x:row r="388">
       <x:c r="A388" s="9"/>
@@ -3918,7 +3528,6 @@
       <x:c r="E388" s="9"/>
       <x:c r="G388" s="9"/>
       <x:c r="H388" s="9"/>
-      <x:c r="K388" s="11"/>
     </x:row>
     <x:row r="389">
       <x:c r="A389" s="9"/>
@@ -3927,7 +3536,6 @@
       <x:c r="E389" s="9"/>
       <x:c r="G389" s="9"/>
       <x:c r="H389" s="9"/>
-      <x:c r="K389" s="11"/>
     </x:row>
     <x:row r="390">
       <x:c r="A390" s="9"/>
@@ -3936,7 +3544,6 @@
       <x:c r="E390" s="9"/>
       <x:c r="G390" s="9"/>
       <x:c r="H390" s="9"/>
-      <x:c r="K390" s="11"/>
     </x:row>
     <x:row r="391">
       <x:c r="A391" s="9"/>
@@ -3945,7 +3552,6 @@
       <x:c r="E391" s="9"/>
       <x:c r="G391" s="9"/>
       <x:c r="H391" s="9"/>
-      <x:c r="K391" s="11"/>
     </x:row>
     <x:row r="392">
       <x:c r="A392" s="9"/>
@@ -3954,7 +3560,6 @@
       <x:c r="E392" s="9"/>
       <x:c r="G392" s="9"/>
       <x:c r="H392" s="9"/>
-      <x:c r="K392" s="11"/>
     </x:row>
     <x:row r="393">
       <x:c r="A393" s="9"/>
@@ -3963,7 +3568,6 @@
       <x:c r="E393" s="9"/>
       <x:c r="G393" s="9"/>
       <x:c r="H393" s="9"/>
-      <x:c r="K393" s="11"/>
     </x:row>
     <x:row r="394">
       <x:c r="A394" s="9"/>
@@ -3972,7 +3576,6 @@
       <x:c r="E394" s="9"/>
       <x:c r="G394" s="9"/>
       <x:c r="H394" s="9"/>
-      <x:c r="K394" s="11"/>
     </x:row>
     <x:row r="395">
       <x:c r="A395" s="9"/>
@@ -3981,7 +3584,6 @@
       <x:c r="E395" s="9"/>
       <x:c r="G395" s="9"/>
       <x:c r="H395" s="9"/>
-      <x:c r="K395" s="11"/>
     </x:row>
     <x:row r="396">
       <x:c r="A396" s="9"/>
@@ -3990,7 +3592,6 @@
       <x:c r="E396" s="9"/>
       <x:c r="G396" s="9"/>
       <x:c r="H396" s="9"/>
-      <x:c r="K396" s="11"/>
     </x:row>
     <x:row r="397">
       <x:c r="A397" s="9"/>
@@ -3999,7 +3600,6 @@
       <x:c r="E397" s="9"/>
       <x:c r="G397" s="9"/>
       <x:c r="H397" s="9"/>
-      <x:c r="K397" s="11"/>
     </x:row>
     <x:row r="398">
       <x:c r="A398" s="9"/>
@@ -4008,7 +3608,6 @@
       <x:c r="E398" s="9"/>
       <x:c r="G398" s="9"/>
       <x:c r="H398" s="9"/>
-      <x:c r="K398" s="11"/>
     </x:row>
     <x:row r="399">
       <x:c r="A399" s="9"/>
@@ -4017,7 +3616,6 @@
       <x:c r="E399" s="9"/>
       <x:c r="G399" s="9"/>
       <x:c r="H399" s="9"/>
-      <x:c r="K399" s="11"/>
     </x:row>
     <x:row r="400">
       <x:c r="A400" s="9"/>
@@ -4026,7 +3624,6 @@
       <x:c r="E400" s="9"/>
       <x:c r="G400" s="9"/>
       <x:c r="H400" s="9"/>
-      <x:c r="K400" s="11"/>
     </x:row>
     <x:row r="401">
       <x:c r="A401" s="9"/>
@@ -4035,7 +3632,6 @@
       <x:c r="E401" s="9"/>
       <x:c r="G401" s="9"/>
       <x:c r="H401" s="9"/>
-      <x:c r="K401" s="11"/>
     </x:row>
     <x:row r="402">
       <x:c r="A402" s="9"/>
@@ -4044,7 +3640,6 @@
       <x:c r="E402" s="9"/>
       <x:c r="G402" s="9"/>
       <x:c r="H402" s="9"/>
-      <x:c r="K402" s="11"/>
     </x:row>
     <x:row r="403">
       <x:c r="A403" s="9"/>
@@ -4053,7 +3648,6 @@
       <x:c r="E403" s="9"/>
       <x:c r="G403" s="9"/>
       <x:c r="H403" s="9"/>
-      <x:c r="K403" s="11"/>
     </x:row>
     <x:row r="404">
       <x:c r="A404" s="9"/>
@@ -4062,7 +3656,6 @@
       <x:c r="E404" s="9"/>
       <x:c r="G404" s="9"/>
       <x:c r="H404" s="9"/>
-      <x:c r="K404" s="11"/>
     </x:row>
     <x:row r="405">
       <x:c r="A405" s="9"/>
@@ -4071,7 +3664,6 @@
       <x:c r="E405" s="9"/>
       <x:c r="G405" s="9"/>
       <x:c r="H405" s="9"/>
-      <x:c r="K405" s="11"/>
     </x:row>
     <x:row r="406">
       <x:c r="A406" s="9"/>
@@ -4080,7 +3672,6 @@
       <x:c r="E406" s="9"/>
       <x:c r="G406" s="9"/>
       <x:c r="H406" s="9"/>
-      <x:c r="K406" s="11"/>
     </x:row>
     <x:row r="407">
       <x:c r="A407" s="9"/>
@@ -4089,7 +3680,6 @@
       <x:c r="E407" s="9"/>
       <x:c r="G407" s="9"/>
       <x:c r="H407" s="9"/>
-      <x:c r="K407" s="11"/>
     </x:row>
     <x:row r="408">
       <x:c r="A408" s="9"/>
@@ -4098,7 +3688,6 @@
       <x:c r="E408" s="9"/>
       <x:c r="G408" s="9"/>
       <x:c r="H408" s="9"/>
-      <x:c r="K408" s="11"/>
     </x:row>
     <x:row r="409">
       <x:c r="A409" s="9"/>
@@ -4107,7 +3696,6 @@
       <x:c r="E409" s="9"/>
       <x:c r="G409" s="9"/>
       <x:c r="H409" s="9"/>
-      <x:c r="K409" s="11"/>
     </x:row>
     <x:row r="410">
       <x:c r="A410" s="9"/>
@@ -4116,7 +3704,6 @@
       <x:c r="E410" s="9"/>
       <x:c r="G410" s="9"/>
       <x:c r="H410" s="9"/>
-      <x:c r="K410" s="11"/>
     </x:row>
     <x:row r="411">
       <x:c r="A411" s="9"/>
@@ -4125,7 +3712,6 @@
       <x:c r="E411" s="9"/>
       <x:c r="G411" s="9"/>
       <x:c r="H411" s="9"/>
-      <x:c r="K411" s="11"/>
     </x:row>
     <x:row r="412">
       <x:c r="A412" s="9"/>
@@ -4134,7 +3720,6 @@
       <x:c r="E412" s="9"/>
       <x:c r="G412" s="9"/>
       <x:c r="H412" s="9"/>
-      <x:c r="K412" s="11"/>
     </x:row>
     <x:row r="413">
       <x:c r="A413" s="9"/>
@@ -4143,7 +3728,6 @@
       <x:c r="E413" s="9"/>
       <x:c r="G413" s="9"/>
       <x:c r="H413" s="9"/>
-      <x:c r="K413" s="11"/>
     </x:row>
     <x:row r="414">
       <x:c r="A414" s="9"/>
@@ -4152,7 +3736,6 @@
       <x:c r="E414" s="9"/>
       <x:c r="G414" s="9"/>
       <x:c r="H414" s="9"/>
-      <x:c r="K414" s="11"/>
     </x:row>
     <x:row r="415">
       <x:c r="A415" s="9"/>
@@ -4161,7 +3744,6 @@
       <x:c r="E415" s="9"/>
       <x:c r="G415" s="9"/>
       <x:c r="H415" s="9"/>
-      <x:c r="K415" s="11"/>
     </x:row>
     <x:row r="416">
       <x:c r="A416" s="9"/>
@@ -4170,7 +3752,6 @@
       <x:c r="E416" s="9"/>
       <x:c r="G416" s="9"/>
       <x:c r="H416" s="9"/>
-      <x:c r="K416" s="11"/>
     </x:row>
     <x:row r="417">
       <x:c r="A417" s="9"/>
@@ -4179,7 +3760,6 @@
       <x:c r="E417" s="9"/>
       <x:c r="G417" s="9"/>
       <x:c r="H417" s="9"/>
-      <x:c r="K417" s="11"/>
     </x:row>
     <x:row r="418">
       <x:c r="A418" s="9"/>
@@ -4188,7 +3768,6 @@
       <x:c r="E418" s="9"/>
       <x:c r="G418" s="9"/>
       <x:c r="H418" s="9"/>
-      <x:c r="K418" s="11"/>
     </x:row>
     <x:row r="419">
       <x:c r="A419" s="9"/>
@@ -4197,7 +3776,6 @@
       <x:c r="E419" s="9"/>
       <x:c r="G419" s="9"/>
       <x:c r="H419" s="9"/>
-      <x:c r="K419" s="11"/>
     </x:row>
     <x:row r="420">
       <x:c r="A420" s="9"/>
@@ -4206,7 +3784,6 @@
       <x:c r="E420" s="9"/>
       <x:c r="G420" s="9"/>
       <x:c r="H420" s="9"/>
-      <x:c r="K420" s="11"/>
     </x:row>
     <x:row r="421">
       <x:c r="A421" s="9"/>
@@ -4215,7 +3792,6 @@
       <x:c r="E421" s="9"/>
       <x:c r="G421" s="9"/>
       <x:c r="H421" s="9"/>
-      <x:c r="K421" s="11"/>
     </x:row>
     <x:row r="422">
       <x:c r="A422" s="9"/>
@@ -4224,7 +3800,6 @@
       <x:c r="E422" s="9"/>
       <x:c r="G422" s="9"/>
       <x:c r="H422" s="9"/>
-      <x:c r="K422" s="11"/>
     </x:row>
     <x:row r="423">
       <x:c r="A423" s="9"/>
@@ -4233,7 +3808,6 @@
       <x:c r="E423" s="9"/>
       <x:c r="G423" s="9"/>
       <x:c r="H423" s="9"/>
-      <x:c r="K423" s="11"/>
     </x:row>
     <x:row r="424">
       <x:c r="A424" s="9"/>
@@ -4242,7 +3816,6 @@
       <x:c r="E424" s="9"/>
       <x:c r="G424" s="9"/>
       <x:c r="H424" s="9"/>
-      <x:c r="K424" s="11"/>
     </x:row>
     <x:row r="425">
       <x:c r="A425" s="9"/>
@@ -4251,7 +3824,6 @@
       <x:c r="E425" s="9"/>
       <x:c r="G425" s="9"/>
       <x:c r="H425" s="9"/>
-      <x:c r="K425" s="11"/>
     </x:row>
     <x:row r="426">
       <x:c r="A426" s="9"/>
@@ -4260,7 +3832,6 @@
       <x:c r="E426" s="9"/>
       <x:c r="G426" s="9"/>
       <x:c r="H426" s="9"/>
-      <x:c r="K426" s="11"/>
     </x:row>
     <x:row r="427">
       <x:c r="A427" s="9"/>
@@ -4269,7 +3840,6 @@
       <x:c r="E427" s="9"/>
       <x:c r="G427" s="9"/>
       <x:c r="H427" s="9"/>
-      <x:c r="K427" s="11"/>
     </x:row>
     <x:row r="428">
       <x:c r="A428" s="9"/>
@@ -4278,7 +3848,6 @@
       <x:c r="E428" s="9"/>
       <x:c r="G428" s="9"/>
       <x:c r="H428" s="9"/>
-      <x:c r="K428" s="11"/>
     </x:row>
     <x:row r="429">
       <x:c r="A429" s="9"/>
@@ -4287,7 +3856,6 @@
       <x:c r="E429" s="9"/>
       <x:c r="G429" s="9"/>
       <x:c r="H429" s="9"/>
-      <x:c r="K429" s="11"/>
     </x:row>
     <x:row r="430">
       <x:c r="A430" s="9"/>
@@ -4296,7 +3864,6 @@
       <x:c r="E430" s="9"/>
       <x:c r="G430" s="9"/>
       <x:c r="H430" s="9"/>
-      <x:c r="K430" s="11"/>
     </x:row>
     <x:row r="431">
       <x:c r="A431" s="9"/>
@@ -4305,7 +3872,6 @@
       <x:c r="E431" s="9"/>
       <x:c r="G431" s="9"/>
       <x:c r="H431" s="9"/>
-      <x:c r="K431" s="11"/>
     </x:row>
     <x:row r="432">
       <x:c r="A432" s="9"/>
@@ -4314,7 +3880,6 @@
       <x:c r="E432" s="9"/>
       <x:c r="G432" s="9"/>
       <x:c r="H432" s="9"/>
-      <x:c r="K432" s="11"/>
     </x:row>
     <x:row r="433">
       <x:c r="A433" s="9"/>
@@ -4323,7 +3888,6 @@
       <x:c r="E433" s="9"/>
       <x:c r="G433" s="9"/>
       <x:c r="H433" s="9"/>
-      <x:c r="K433" s="11"/>
     </x:row>
     <x:row r="434">
       <x:c r="A434" s="9"/>
@@ -4332,7 +3896,6 @@
       <x:c r="E434" s="9"/>
       <x:c r="G434" s="9"/>
       <x:c r="H434" s="9"/>
-      <x:c r="K434" s="11"/>
     </x:row>
     <x:row r="435">
       <x:c r="A435" s="9"/>
@@ -4341,7 +3904,6 @@
       <x:c r="E435" s="9"/>
       <x:c r="G435" s="9"/>
       <x:c r="H435" s="9"/>
-      <x:c r="K435" s="11"/>
     </x:row>
     <x:row r="436">
       <x:c r="A436" s="9"/>
@@ -4350,7 +3912,6 @@
       <x:c r="E436" s="9"/>
       <x:c r="G436" s="9"/>
       <x:c r="H436" s="9"/>
-      <x:c r="K436" s="11"/>
     </x:row>
     <x:row r="437">
       <x:c r="A437" s="9"/>
@@ -4359,7 +3920,6 @@
       <x:c r="E437" s="9"/>
       <x:c r="G437" s="9"/>
       <x:c r="H437" s="9"/>
-      <x:c r="K437" s="11"/>
     </x:row>
     <x:row r="438">
       <x:c r="A438" s="9"/>
@@ -4368,7 +3928,6 @@
       <x:c r="E438" s="9"/>
       <x:c r="G438" s="9"/>
       <x:c r="H438" s="9"/>
-      <x:c r="K438" s="11"/>
     </x:row>
     <x:row r="439">
       <x:c r="A439" s="9"/>
@@ -4377,7 +3936,6 @@
       <x:c r="E439" s="9"/>
       <x:c r="G439" s="9"/>
       <x:c r="H439" s="9"/>
-      <x:c r="K439" s="11"/>
     </x:row>
     <x:row r="440">
       <x:c r="A440" s="9"/>
@@ -4386,7 +3944,6 @@
       <x:c r="E440" s="9"/>
       <x:c r="G440" s="9"/>
       <x:c r="H440" s="9"/>
-      <x:c r="K440" s="11"/>
     </x:row>
     <x:row r="441">
       <x:c r="A441" s="9"/>
@@ -4395,7 +3952,6 @@
       <x:c r="E441" s="9"/>
       <x:c r="G441" s="9"/>
       <x:c r="H441" s="9"/>
-      <x:c r="K441" s="11"/>
     </x:row>
     <x:row r="442">
       <x:c r="A442" s="9"/>
@@ -4404,7 +3960,6 @@
       <x:c r="E442" s="9"/>
       <x:c r="G442" s="9"/>
       <x:c r="H442" s="9"/>
-      <x:c r="K442" s="11"/>
     </x:row>
     <x:row r="443">
       <x:c r="A443" s="9"/>
@@ -4413,7 +3968,6 @@
       <x:c r="E443" s="9"/>
       <x:c r="G443" s="9"/>
       <x:c r="H443" s="9"/>
-      <x:c r="K443" s="11"/>
     </x:row>
     <x:row r="444">
       <x:c r="A444" s="9"/>
@@ -4422,7 +3976,6 @@
       <x:c r="E444" s="9"/>
       <x:c r="G444" s="9"/>
       <x:c r="H444" s="9"/>
-      <x:c r="K444" s="11"/>
     </x:row>
     <x:row r="445">
       <x:c r="A445" s="9"/>
@@ -4431,7 +3984,6 @@
       <x:c r="E445" s="9"/>
       <x:c r="G445" s="9"/>
       <x:c r="H445" s="9"/>
-      <x:c r="K445" s="11"/>
     </x:row>
     <x:row r="446">
       <x:c r="A446" s="9"/>
@@ -4440,7 +3992,6 @@
       <x:c r="E446" s="9"/>
       <x:c r="G446" s="9"/>
       <x:c r="H446" s="9"/>
-      <x:c r="K446" s="11"/>
     </x:row>
     <x:row r="447">
       <x:c r="A447" s="9"/>
@@ -4449,7 +4000,6 @@
       <x:c r="E447" s="9"/>
       <x:c r="G447" s="9"/>
       <x:c r="H447" s="9"/>
-      <x:c r="K447" s="11"/>
     </x:row>
     <x:row r="448">
       <x:c r="A448" s="9"/>
@@ -4458,7 +4008,6 @@
       <x:c r="E448" s="9"/>
       <x:c r="G448" s="9"/>
       <x:c r="H448" s="9"/>
-      <x:c r="K448" s="11"/>
     </x:row>
     <x:row r="449">
       <x:c r="A449" s="9"/>
@@ -4467,7 +4016,6 @@
       <x:c r="E449" s="9"/>
       <x:c r="G449" s="9"/>
       <x:c r="H449" s="9"/>
-      <x:c r="K449" s="11"/>
     </x:row>
     <x:row r="450">
       <x:c r="A450" s="9"/>
@@ -4476,7 +4024,6 @@
       <x:c r="E450" s="9"/>
       <x:c r="G450" s="9"/>
       <x:c r="H450" s="9"/>
-      <x:c r="K450" s="11"/>
     </x:row>
     <x:row r="451">
       <x:c r="A451" s="9"/>
@@ -4485,7 +4032,6 @@
       <x:c r="E451" s="9"/>
       <x:c r="G451" s="9"/>
       <x:c r="H451" s="9"/>
-      <x:c r="K451" s="11"/>
     </x:row>
     <x:row r="452">
       <x:c r="A452" s="9"/>
@@ -4494,7 +4040,6 @@
       <x:c r="E452" s="9"/>
       <x:c r="G452" s="9"/>
       <x:c r="H452" s="9"/>
-      <x:c r="K452" s="11"/>
     </x:row>
     <x:row r="453">
       <x:c r="A453" s="9"/>
@@ -4503,7 +4048,6 @@
       <x:c r="E453" s="9"/>
       <x:c r="G453" s="9"/>
       <x:c r="H453" s="9"/>
-      <x:c r="K453" s="11"/>
     </x:row>
     <x:row r="454">
       <x:c r="A454" s="9"/>
@@ -4512,7 +4056,6 @@
       <x:c r="E454" s="9"/>
       <x:c r="G454" s="9"/>
       <x:c r="H454" s="9"/>
-      <x:c r="K454" s="11"/>
     </x:row>
     <x:row r="455">
       <x:c r="A455" s="9"/>
@@ -4521,7 +4064,6 @@
       <x:c r="E455" s="9"/>
       <x:c r="G455" s="9"/>
       <x:c r="H455" s="9"/>
-      <x:c r="K455" s="11"/>
     </x:row>
     <x:row r="456">
       <x:c r="A456" s="9"/>
@@ -4530,7 +4072,6 @@
       <x:c r="E456" s="9"/>
       <x:c r="G456" s="9"/>
       <x:c r="H456" s="9"/>
-      <x:c r="K456" s="11"/>
     </x:row>
     <x:row r="457">
       <x:c r="A457" s="9"/>
@@ -4539,7 +4080,6 @@
       <x:c r="E457" s="9"/>
       <x:c r="G457" s="9"/>
       <x:c r="H457" s="9"/>
-      <x:c r="K457" s="11"/>
     </x:row>
     <x:row r="458">
       <x:c r="A458" s="9"/>
@@ -4548,7 +4088,6 @@
       <x:c r="E458" s="9"/>
       <x:c r="G458" s="9"/>
       <x:c r="H458" s="9"/>
-      <x:c r="K458" s="11"/>
     </x:row>
     <x:row r="459">
       <x:c r="A459" s="9"/>
@@ -4557,7 +4096,6 @@
       <x:c r="E459" s="9"/>
       <x:c r="G459" s="9"/>
       <x:c r="H459" s="9"/>
-      <x:c r="K459" s="11"/>
     </x:row>
     <x:row r="460">
       <x:c r="A460" s="9"/>
@@ -4566,7 +4104,6 @@
       <x:c r="E460" s="9"/>
       <x:c r="G460" s="9"/>
       <x:c r="H460" s="9"/>
-      <x:c r="K460" s="11"/>
     </x:row>
     <x:row r="461">
       <x:c r="A461" s="9"/>
@@ -4575,7 +4112,6 @@
       <x:c r="E461" s="9"/>
       <x:c r="G461" s="9"/>
       <x:c r="H461" s="9"/>
-      <x:c r="K461" s="11"/>
     </x:row>
     <x:row r="462">
       <x:c r="A462" s="9"/>
@@ -4584,7 +4120,6 @@
       <x:c r="E462" s="9"/>
       <x:c r="G462" s="9"/>
       <x:c r="H462" s="9"/>
-      <x:c r="K462" s="11"/>
     </x:row>
     <x:row r="463">
       <x:c r="A463" s="9"/>
@@ -4593,7 +4128,6 @@
       <x:c r="E463" s="9"/>
       <x:c r="G463" s="9"/>
       <x:c r="H463" s="9"/>
-      <x:c r="K463" s="11"/>
     </x:row>
     <x:row r="464">
       <x:c r="A464" s="9"/>
@@ -4602,7 +4136,6 @@
       <x:c r="E464" s="9"/>
       <x:c r="G464" s="9"/>
       <x:c r="H464" s="9"/>
-      <x:c r="K464" s="11"/>
     </x:row>
     <x:row r="465">
       <x:c r="A465" s="9"/>
@@ -4611,7 +4144,6 @@
       <x:c r="E465" s="9"/>
       <x:c r="G465" s="9"/>
       <x:c r="H465" s="9"/>
-      <x:c r="K465" s="11"/>
     </x:row>
     <x:row r="466">
       <x:c r="A466" s="9"/>
@@ -4620,7 +4152,6 @@
       <x:c r="E466" s="9"/>
       <x:c r="G466" s="9"/>
       <x:c r="H466" s="9"/>
-      <x:c r="K466" s="11"/>
     </x:row>
     <x:row r="467">
       <x:c r="A467" s="9"/>
@@ -4629,7 +4160,6 @@
       <x:c r="E467" s="9"/>
       <x:c r="G467" s="9"/>
       <x:c r="H467" s="9"/>
-      <x:c r="K467" s="11"/>
     </x:row>
     <x:row r="468">
       <x:c r="A468" s="9"/>
@@ -4638,7 +4168,6 @@
       <x:c r="E468" s="9"/>
       <x:c r="G468" s="9"/>
       <x:c r="H468" s="9"/>
-      <x:c r="K468" s="11"/>
     </x:row>
     <x:row r="469">
       <x:c r="A469" s="9"/>
@@ -4647,7 +4176,6 @@
       <x:c r="E469" s="9"/>
       <x:c r="G469" s="9"/>
       <x:c r="H469" s="9"/>
-      <x:c r="K469" s="11"/>
     </x:row>
     <x:row r="470">
       <x:c r="A470" s="9"/>
@@ -4656,7 +4184,6 @@
       <x:c r="E470" s="9"/>
       <x:c r="G470" s="9"/>
       <x:c r="H470" s="9"/>
-      <x:c r="K470" s="11"/>
     </x:row>
     <x:row r="471">
       <x:c r="A471" s="9"/>
@@ -4665,7 +4192,6 @@
       <x:c r="E471" s="9"/>
       <x:c r="G471" s="9"/>
       <x:c r="H471" s="9"/>
-      <x:c r="K471" s="11"/>
     </x:row>
     <x:row r="472">
       <x:c r="A472" s="9"/>
@@ -4674,7 +4200,6 @@
       <x:c r="E472" s="9"/>
       <x:c r="G472" s="9"/>
       <x:c r="H472" s="9"/>
-      <x:c r="K472" s="11"/>
     </x:row>
     <x:row r="473">
       <x:c r="A473" s="9"/>
@@ -4683,7 +4208,6 @@
       <x:c r="E473" s="9"/>
       <x:c r="G473" s="9"/>
       <x:c r="H473" s="9"/>
-      <x:c r="K473" s="11"/>
     </x:row>
     <x:row r="474">
       <x:c r="A474" s="9"/>
@@ -4692,7 +4216,6 @@
       <x:c r="E474" s="9"/>
       <x:c r="G474" s="9"/>
       <x:c r="H474" s="9"/>
-      <x:c r="K474" s="11"/>
     </x:row>
     <x:row r="475">
       <x:c r="A475" s="9"/>
@@ -4701,7 +4224,6 @@
       <x:c r="E475" s="9"/>
       <x:c r="G475" s="9"/>
       <x:c r="H475" s="9"/>
-      <x:c r="K475" s="11"/>
     </x:row>
     <x:row r="476">
       <x:c r="A476" s="9"/>
@@ -4710,7 +4232,6 @@
       <x:c r="E476" s="9"/>
       <x:c r="G476" s="9"/>
       <x:c r="H476" s="9"/>
-      <x:c r="K476" s="11"/>
     </x:row>
     <x:row r="477">
       <x:c r="A477" s="9"/>
@@ -4719,7 +4240,6 @@
       <x:c r="E477" s="9"/>
       <x:c r="G477" s="9"/>
       <x:c r="H477" s="9"/>
-      <x:c r="K477" s="11"/>
     </x:row>
     <x:row r="478">
       <x:c r="A478" s="9"/>
@@ -4728,7 +4248,6 @@
       <x:c r="E478" s="9"/>
       <x:c r="G478" s="9"/>
       <x:c r="H478" s="9"/>
-      <x:c r="K478" s="11"/>
     </x:row>
     <x:row r="479">
       <x:c r="A479" s="9"/>
@@ -4737,7 +4256,6 @@
       <x:c r="E479" s="9"/>
       <x:c r="G479" s="9"/>
       <x:c r="H479" s="9"/>
-      <x:c r="K479" s="11"/>
     </x:row>
     <x:row r="480">
       <x:c r="A480" s="9"/>
@@ -4746,7 +4264,6 @@
       <x:c r="E480" s="9"/>
       <x:c r="G480" s="9"/>
       <x:c r="H480" s="9"/>
-      <x:c r="K480" s="11"/>
     </x:row>
     <x:row r="481">
       <x:c r="A481" s="9"/>
@@ -4755,7 +4272,6 @@
       <x:c r="E481" s="9"/>
       <x:c r="G481" s="9"/>
       <x:c r="H481" s="9"/>
-      <x:c r="K481" s="11"/>
     </x:row>
     <x:row r="482">
       <x:c r="A482" s="9"/>
@@ -4764,7 +4280,6 @@
       <x:c r="E482" s="9"/>
       <x:c r="G482" s="9"/>
       <x:c r="H482" s="9"/>
-      <x:c r="K482" s="11"/>
     </x:row>
     <x:row r="483">
       <x:c r="A483" s="9"/>
@@ -4773,7 +4288,6 @@
       <x:c r="E483" s="9"/>
       <x:c r="G483" s="9"/>
       <x:c r="H483" s="9"/>
-      <x:c r="K483" s="11"/>
     </x:row>
     <x:row r="484">
       <x:c r="A484" s="9"/>
@@ -4782,7 +4296,6 @@
       <x:c r="E484" s="9"/>
       <x:c r="G484" s="9"/>
       <x:c r="H484" s="9"/>
-      <x:c r="K484" s="11"/>
     </x:row>
     <x:row r="485">
       <x:c r="A485" s="9"/>
@@ -4791,7 +4304,6 @@
       <x:c r="E485" s="9"/>
       <x:c r="G485" s="9"/>
       <x:c r="H485" s="9"/>
-      <x:c r="K485" s="11"/>
     </x:row>
     <x:row r="486">
       <x:c r="A486" s="9"/>
@@ -4800,7 +4312,6 @@
       <x:c r="E486" s="9"/>
       <x:c r="G486" s="9"/>
       <x:c r="H486" s="9"/>
-      <x:c r="K486" s="11"/>
     </x:row>
     <x:row r="487">
       <x:c r="A487" s="9"/>
@@ -4809,7 +4320,6 @@
       <x:c r="E487" s="9"/>
       <x:c r="G487" s="9"/>
       <x:c r="H487" s="9"/>
-      <x:c r="K487" s="11"/>
     </x:row>
     <x:row r="488">
       <x:c r="A488" s="9"/>
@@ -4818,7 +4328,6 @@
       <x:c r="E488" s="9"/>
       <x:c r="G488" s="9"/>
       <x:c r="H488" s="9"/>
-      <x:c r="K488" s="11"/>
     </x:row>
     <x:row r="489">
       <x:c r="A489" s="9"/>
@@ -4827,7 +4336,6 @@
       <x:c r="E489" s="9"/>
       <x:c r="G489" s="9"/>
       <x:c r="H489" s="9"/>
-      <x:c r="K489" s="11"/>
     </x:row>
     <x:row r="490">
       <x:c r="A490" s="9"/>
@@ -4836,7 +4344,6 @@
       <x:c r="E490" s="9"/>
       <x:c r="G490" s="9"/>
       <x:c r="H490" s="9"/>
-      <x:c r="K490" s="11"/>
     </x:row>
     <x:row r="491">
       <x:c r="A491" s="9"/>
@@ -4845,7 +4352,6 @@
       <x:c r="E491" s="9"/>
       <x:c r="G491" s="9"/>
       <x:c r="H491" s="9"/>
-      <x:c r="K491" s="11"/>
     </x:row>
     <x:row r="492">
       <x:c r="A492" s="9"/>
@@ -4854,7 +4360,6 @@
       <x:c r="E492" s="9"/>
       <x:c r="G492" s="9"/>
       <x:c r="H492" s="9"/>
-      <x:c r="K492" s="11"/>
     </x:row>
     <x:row r="493">
       <x:c r="A493" s="9"/>
@@ -4863,7 +4368,6 @@
       <x:c r="E493" s="9"/>
       <x:c r="G493" s="9"/>
       <x:c r="H493" s="9"/>
-      <x:c r="K493" s="11"/>
     </x:row>
     <x:row r="494">
       <x:c r="A494" s="9"/>
@@ -4872,7 +4376,6 @@
       <x:c r="E494" s="9"/>
       <x:c r="G494" s="9"/>
       <x:c r="H494" s="9"/>
-      <x:c r="K494" s="11"/>
     </x:row>
     <x:row r="495">
       <x:c r="A495" s="9"/>
@@ -4881,7 +4384,6 @@
       <x:c r="E495" s="9"/>
       <x:c r="G495" s="9"/>
       <x:c r="H495" s="9"/>
-      <x:c r="K495" s="11"/>
     </x:row>
     <x:row r="496">
       <x:c r="A496" s="9"/>
@@ -4890,7 +4392,6 @@
       <x:c r="E496" s="9"/>
       <x:c r="G496" s="9"/>
       <x:c r="H496" s="9"/>
-      <x:c r="K496" s="11"/>
     </x:row>
     <x:row r="497">
       <x:c r="A497" s="9"/>
@@ -4899,7 +4400,6 @@
       <x:c r="E497" s="9"/>
       <x:c r="G497" s="9"/>
       <x:c r="H497" s="9"/>
-      <x:c r="K497" s="11"/>
     </x:row>
     <x:row r="498">
       <x:c r="A498" s="9"/>
@@ -4908,7 +4408,6 @@
       <x:c r="E498" s="9"/>
       <x:c r="G498" s="9"/>
       <x:c r="H498" s="9"/>
-      <x:c r="K498" s="11"/>
     </x:row>
     <x:row r="499">
       <x:c r="A499" s="9"/>
@@ -4917,7 +4416,6 @@
       <x:c r="E499" s="9"/>
       <x:c r="G499" s="9"/>
       <x:c r="H499" s="9"/>
-      <x:c r="K499" s="11"/>
     </x:row>
     <x:row r="500">
       <x:c r="A500" s="9"/>
@@ -4926,7 +4424,6 @@
       <x:c r="E500" s="9"/>
       <x:c r="G500" s="9"/>
       <x:c r="H500" s="9"/>
-      <x:c r="K500" s="11"/>
     </x:row>
     <x:row r="501">
       <x:c r="A501" s="9"/>
@@ -4935,7 +4432,6 @@
       <x:c r="E501" s="9"/>
       <x:c r="G501" s="9"/>
       <x:c r="H501" s="9"/>
-      <x:c r="K501" s="11"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5043,7 +4539,7 @@
         <x:v>گارانتی</x:v>
       </x:c>
       <x:c r="B12" s="13" t="str">
-        <x:v>این فرم گارانتی را فعال نمی‌کند و تاریخ شروع گارانتی را تغییر نمی‌دهد.</x:v>
+        <x:v>تاریخ فعال‌سازی از اولین صدور موفق کد در نرم‌افزار ثبت می‌شود و ستون ورودی اکسل ندارد.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">

</xml_diff>